<commit_message>
feat(F-NAR-016): TREE-DIF-029 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-029.xlsx
+++ b/stories/arbres/TREE-DIF-029.xlsx
@@ -1933,12 +1933,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le sac porte le filet, tout contre le tissu. Il est trop vert ! C'est pour faire de l'ombre. Aniss a les genoux plus bas que Victorino. Ses pieds n'arrêtent pas de bouger. Il a beaucoup d'élan, ce n'est rien. On reste près des champs ? Oui, papa.</t>
+          <t>Le sac tient le filet, tout près de la hanche. On dirait une fenêtre verte ! Le jaune aime l'ombre, un peu. Aniss avance, recule, avance encore. Ses lacets n'ont pas le temps de pendre. Il a envie de courir, on le voit. Le pré est juste derrière le portail ? Oui, papa.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le sac porte le filet, tout contre le tissu. Il est trop vert ! C'est pour faire de l'ombre. Aniss a les genoux plus bas que Victorino. Ses pieds n'arrêtent pas de bouger. Il a beaucoup d'élan, ce n'est rien. On reste près des champs ? Oui, papa.</t>
+          <t>Le sac tient le filet, tout près de la hanche. On dirait une fenêtre verte ! Le jaune aime l'ombre, un peu. Aniss avance, recule, avance encore. Ses lacets n'ont pas le temps de pendre. Il a envie de courir, on le voit. Le pré est juste derrière le portail ? Oui, papa.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2077,13 +2077,13 @@
       </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le sac porte le filet, tout contre le tissu.
-copain|Il est trop vert !
-enfant-m|C'est pour faire de l'ombre.
-narrateur|Aniss a les genoux plus bas que Victorino.
-narrateur|Ses pieds n'arrêtent pas de bouger.
-maman|Il a beaucoup d'élan, ce n'est rien.
-papa|On reste près des champs ?
+          <t>narrateur|Le sac tient le filet, tout près de la hanche.
+copain|On dirait une fenêtre verte !
+enfant-m|Le jaune aime l'ombre, un peu.
+narrateur|Aniss avance, recule, avance encore.
+narrateur|Ses lacets n'ont pas le temps de pendre.
+maman|Il a envie de courir, on le voit.
+papa|Le pré est juste derrière le portail ?
 enfant-m|Oui, papa.</t>
         </is>
       </c>
@@ -2111,12 +2111,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Aniss tapote déjà le sol, tout léger. Le pré a l'herbe haute, encore tiède. Les lavandes sentent fort, tout bas. Le muret garde une pierre chaude. On commence où, pour le papillon ?</t>
+          <t>Aniss tape déjà deux cailloux, l'un contre l'autre. Le pré ondule, plus loin que le puits. Les lavandes font un mur violet, tout bas. Le muret tient encore la chaleur du chat. On guette où, d'abord ?</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Aniss tapote déjà le sol, tout léger. Le pré a l'herbe haute, encore tiède. Les lavandes sentent fort, tout bas. Le muret garde une pierre chaude. On commence où, pour le papillon ?</t>
+          <t>Aniss tape déjà deux cailloux, l'un contre l'autre. Le pré ondule, plus loin que le puits. Les lavandes font un mur violet, tout bas. Le muret tient encore la chaleur du chat. On guette où, d'abord ?</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -2275,11 +2275,11 @@
       <c r="AV7" s="2" t="inlineStr"/>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>narrateur|Aniss tapote déjà le sol, tout léger.
-narrateur|Le pré a l'herbe haute, encore tiède.
-narrateur|Les lavandes sentent fort, tout bas.
-narrateur|Le muret garde une pierre chaude.
-papa|On commence où, pour le papillon ?</t>
+          <t>narrateur|Aniss tape déjà deux cailloux, l'un contre l'autre.
+narrateur|Le pré ondule, plus loin que le puits.
+narrateur|Les lavandes font un mur violet, tout bas.
+narrateur|Le muret tient encore la chaleur du chat.
+papa|On guette où, d'abord ?</t>
         </is>
       </c>
     </row>
@@ -2306,12 +2306,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Victorino lève le filet, comme un toit. L'herbe du pré sent le foin chaud. Moi je cours, Victorino ! Aniss fend l'herbe, trop vite. Un nuage de graines s'envole, tout haut. Le filet racle l'herbe, trop vite. Le filet vert n'attendait pas ça. Il a envie de bouger, c'est tout. Ses jambes sont plus courtes, plus vives. On guette comment, alors ? Vous faites comment, tous les deux ?</t>
+          <t>Victorino lève le filet, comme un toit. Les tiges se touchent, puis se séparent. Je le rattrape ! Aniss part dans l'herbe, trop loin. Le jaune s'envole, plus haut que leurs têtes. Le filet racle l'herbe, trop vite. Le filet vert n'a pas suffi. Il a envie de courir, c'est tout. Tes pieds vont trop vite, Aniss. Je fais comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Victorino lève le filet, comme un toit. L'herbe du pré sent le foin chaud. Moi je cours, Victorino ! Aniss fend l'herbe, trop vite. Un nuage de graines s'envole, tout haut. Le filet racle l'herbe, trop vite. Le filet vert n'attendait pas ça. Il a envie de bouger, c'est tout. Ses jambes sont plus courtes, plus vives. On guette comment, alors ? Vous faites comment, tous les deux ?</t>
+          <t>Victorino lève le filet, comme un toit. Les tiges se touchent, puis se séparent. Je le rattrape ! Aniss part dans l'herbe, trop loin. Le jaune s'envole, plus haut que leurs têtes. Le filet racle l'herbe, trop vite. Le filet vert n'a pas suffi. Il a envie de courir, c'est tout. Tes pieds vont trop vite, Aniss. Je fais comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -2447,16 +2447,16 @@
       <c r="AW8" t="inlineStr">
         <is>
           <t>narrateur|Victorino lève le filet, comme un toit.
-narrateur|L'herbe du pré sent le foin chaud.
-copain|Moi je cours, Victorino !
-narrateur|Aniss fend l'herbe, trop vite.
-narrateur|Un nuage de graines s'envole, tout haut.
+narrateur|Les tiges se touchent, puis se séparent.
+copain|Je le rattrape !
+narrateur|Aniss part dans l'herbe, trop loin.
+narrateur|Le jaune s'envole, plus haut que leurs têtes.
 narrateur|Le filet racle l'herbe, trop vite.
-enfant-m|Le filet vert n'attendait pas ça.
-maman|Il a envie de bouger, c'est tout.
-papa|Ses jambes sont plus courtes, plus vives.
-copain|On guette comment, alors ?
-papa|Vous faites comment, tous les deux ?</t>
+enfant-m|Le filet vert n'a pas suffi.
+maman|Il a envie de courir, c'est tout.
+papa|Tes pieds vont trop vite, Aniss.
+copain|Je fais comment, alors ?
+papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="AX8" t="inlineStr">
@@ -2488,12 +2488,12 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Aniss fend encore l'herbe, tout léger. Marcher comme lui, s'asseoir, ou maman ?</t>
+          <t>L'herbe se referme derrière Aniss. Marcher comme lui, s'asseoir, ou le silence ?</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Aniss fend encore l'herbe, tout léger. Marcher comme lui, s'asseoir, ou maman ?</t>
+          <t>L'herbe se referme derrière Aniss. Marcher comme lui, s'asseoir, ou le silence ?</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -2652,8 +2652,8 @@
       <c r="AV9" s="2" t="inlineStr"/>
       <c r="AW9" t="inlineStr">
         <is>
-          <t>narrateur|Aniss fend encore l'herbe, tout léger.
-papa|Marcher comme lui, s'asseoir, ou maman ?</t>
+          <t>narrateur|L'herbe se referme derrière Aniss.
+papa|Marcher comme lui, s'asseoir, ou le silence ?</t>
         </is>
       </c>
     </row>
@@ -2680,12 +2680,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>On marche comme lui. Moi je bats des bras, tout lent. Aniss tient le sac, Victorino lève le filet. Deux ombres avancent dans l'herbe, sans courir. Aniss lève un pied, puis s'arrête. Maintenant c'est moi. Puis c'est moi encore. Vous jouez à son pas. L'élan a trouvé sa place.</t>
+          <t>On marche comme lui. Moi je bats des bras, tout lent. Le filet suit leurs bras, tout lent. Deux ombres avancent dans l'herbe, sans courir. Aniss lève un pied, puis le repose. Le jaune a des ailes comme ça. Les miennes aussi, maintenant. Vous jouez à son pas. Le pré vous a laissés entrer.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>On marche comme lui. Moi je bats des bras, tout lent. Aniss tient le sac, Victorino lève le filet. Deux ombres avancent dans l'herbe, sans courir. Aniss lève un pied, puis s'arrête. Maintenant c'est moi. Puis c'est moi encore. Vous jouez à son pas. L'élan a trouvé sa place.</t>
+          <t>On marche comme lui. Moi je bats des bras, tout lent. Le filet suit leurs bras, tout lent. Deux ombres avancent dans l'herbe, sans courir. Aniss lève un pied, puis le repose. Le jaune a des ailes comme ça. Les miennes aussi, maintenant. Vous jouez à son pas. Le pré vous a laissés entrer.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -2822,13 +2822,13 @@
         <is>
           <t>enfant-m|On marche comme lui.
 copain|Moi je bats des bras, tout lent.
-narrateur|Aniss tient le sac, Victorino lève le filet.
+narrateur|Le filet suit leurs bras, tout lent.
 narrateur|Deux ombres avancent dans l'herbe, sans courir.
-narrateur|Aniss lève un pied, puis s'arrête.
-enfant-m|Maintenant c'est moi.
-copain|Puis c'est moi encore.
+narrateur|Aniss lève un pied, puis le repose.
+enfant-m|Le jaune a des ailes comme ça.
+copain|Les miennes aussi, maintenant.
 papa|Vous jouez à son pas.
-maman|L'élan a trouvé sa place.</t>
+maman|Le pré vous a laissés entrer.</t>
         </is>
       </c>
     </row>
@@ -2855,12 +2855,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Le papillon jaune se pose, au bout d'une tige. On a marché, chacun son tour. Tu battais des bras, moi j'avançais. Vous avez laissé l'élan dessiner. Le pré sent encore le foin. Le filet vert rentre dans le sac. Une poudre jaune dort sur l'herbe. On rentre, Aniss. Le portail de bois cliquette, tout seul.</t>
+          <t>Le papillon jaune se pose, au bout d'une tige. Mes bras ont fait des ailes. Les miennes aussi, tout lent. Vous avez marché à son pas. Le pré sent encore le foin. Le filet vert rentre dans le sac. Une poudre jaune dort sur l'herbe. Il est venu, Aniss. Le portail de bois cliquette, tout seul.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Le papillon jaune se pose, au bout d'une tige. On a marché, chacun son tour. Tu battais des bras, moi j'avançais. Vous avez laissé l'élan dessiner. Le pré sent encore le foin. Le filet vert rentre dans le sac. Une poudre jaune dort sur l'herbe. On rentre, Aniss. Le portail de bois cliquette, tout seul.</t>
+          <t>Le papillon jaune se pose, au bout d'une tige. Mes bras ont fait des ailes. Les miennes aussi, tout lent. Vous avez marché à son pas. Le pré sent encore le foin. Le filet vert rentre dans le sac. Une poudre jaune dort sur l'herbe. Il est venu, Aniss. Le portail de bois cliquette, tout seul.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2996,13 +2996,13 @@
       <c r="AW11" t="inlineStr">
         <is>
           <t>narrateur|Le papillon jaune se pose, au bout d'une tige.
-copain|On a marché, chacun son tour.
-enfant-m|Tu battais des bras, moi j'avançais.
-papa|Vous avez laissé l'élan dessiner.
+copain|Mes bras ont fait des ailes.
+enfant-m|Les miennes aussi, tout lent.
+papa|Vous avez marché à son pas.
 maman|Le pré sent encore le foin.
 narrateur|Le filet vert rentre dans le sac.
 narrateur|Une poudre jaune dort sur l'herbe.
-enfant-m|On rentre, Aniss.
+enfant-m|Il est venu, Aniss.
 narrateur|Le portail de bois cliquette, tout seul.</t>
         </is>
       </c>
@@ -3030,12 +3030,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>On s'assoit un peu. Je m'assois, alors. Aniss pose les genoux dans l'herbe. Le filet vert attend près des genoux. Sa respiration redevient calme, tout doux. Tu es prêt ? Je ne cours plus. Vous avez laissé l'élan s'asseoir. Le pré vous a gardés.</t>
+          <t>On s'assoit un peu. Je m'assois, alors. Aniss pose les genoux dans l'herbe. Le filet vert dort sur les genoux. Une tige se redresse, tout contre sa chaussure. Tu es prêt ? Je ne cours plus. Vous avez attendu l'herbe. Le jaune peut redescendre, maintenant.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>On s'assoit un peu. Je m'assois, alors. Aniss pose les genoux dans l'herbe. Le filet vert attend près des genoux. Sa respiration redevient calme, tout doux. Tu es prêt ? Je ne cours plus. Vous avez laissé l'élan s'asseoir. Le pré vous a gardés.</t>
+          <t>On s'assoit un peu. Je m'assois, alors. Aniss pose les genoux dans l'herbe. Le filet vert dort sur les genoux. Une tige se redresse, tout contre sa chaussure. Tu es prêt ? Je ne cours plus. Vous avez attendu l'herbe. Le jaune peut redescendre, maintenant.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -3173,12 +3173,12 @@
           <t>enfant-m|On s'assoit un peu.
 copain|Je m'assois, alors.
 narrateur|Aniss pose les genoux dans l'herbe.
-narrateur|Le filet vert attend près des genoux.
-narrateur|Sa respiration redevient calme, tout doux.
+narrateur|Le filet vert dort sur les genoux.
+narrateur|Une tige se redresse, tout contre sa chaussure.
 enfant-m|Tu es prêt ?
 copain|Je ne cours plus.
-papa|Vous avez laissé l'élan s'asseoir.
-maman|Le pré vous a gardés.</t>
+papa|Vous avez attendu l'herbe.
+maman|Le jaune peut redescendre, maintenant.</t>
         </is>
       </c>
     </row>
@@ -3205,12 +3205,12 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>L'herbe garde encore la chaleur des genoux. Tu t'es assis, d'abord. Puis le jaune est venu, tout droit. L'élan s'est assis, puis il a guetté. Le pré redevient calme. Le filet vert rentre dans le sac. Une graine reste coincée au tissu. À demain, les tiges. Le gravier du chemin brille un peu.</t>
+          <t>L'herbe garde encore la chaleur des genoux. Tu t'es assis, d'abord. Puis le jaune est venu, tout droit. Vous avez attendu, assis. Une tige vous a chatouillés, sans rien dire. Le filet vert rentre dans le sac. Une graine reste coincée au tissu. À demain, les tiges. Le gravier du chemin brille un peu.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>L'herbe garde encore la chaleur des genoux. Tu t'es assis, d'abord. Puis le jaune est venu, tout droit. L'élan s'est assis, puis il a guetté. Le pré redevient calme. Le filet vert rentre dans le sac. Une graine reste coincée au tissu. À demain, les tiges. Le gravier du chemin brille un peu.</t>
+          <t>L'herbe garde encore la chaleur des genoux. Tu t'es assis, d'abord. Puis le jaune est venu, tout droit. Vous avez attendu, assis. Une tige vous a chatouillés, sans rien dire. Le filet vert rentre dans le sac. Une graine reste coincée au tissu. À demain, les tiges. Le gravier du chemin brille un peu.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -3348,8 +3348,8 @@
           <t>narrateur|L'herbe garde encore la chaleur des genoux.
 enfant-m|Tu t'es assis, d'abord.
 copain|Puis le jaune est venu, tout droit.
-papa|L'élan s'est assis, puis il a guetté.
-maman|Le pré redevient calme.
+papa|Vous avez attendu, assis.
+maman|Une tige vous a chatouillés, sans rien dire.
 narrateur|Le filet vert rentre dans le sac.
 narrateur|Une graine reste coincée au tissu.
 enfant-m|À demain, les tiges.
@@ -3380,12 +3380,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu restes avec nous ? Un, deux, trois, on ne bouge plus. Aniss s'arrête seulement quand elle dit trois. Victorino lève le filet à chaque chiffre. Je peux attendre le trois ! Moi aussi, j'attends. L'herbe redevient droite, autour. Vous avez demandé, et ça marche. Mes chiffres ont tenu l'élan.</t>
+          <t>Maman, tu restes avec nous ? Chut, on écoute l'herbe. Aniss ouvre la bouche, puis la referme. Victorino tient le filet, sans le secouer. Je peux être silencieux ! Moi aussi, j'écoute. Un criquet reprend, tout près. Vous avez demandé, et ça tient. Mon chut a tenu vos pieds.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu restes avec nous ? Un, deux, trois, on ne bouge plus. Aniss s'arrête seulement quand elle dit trois. Victorino lève le filet à chaque chiffre. Je peux attendre le trois ! Moi aussi, j'attends. L'herbe redevient droite, autour. Vous avez demandé, et ça marche. Mes chiffres ont tenu l'élan.</t>
+          <t>Maman, tu restes avec nous ? Chut, on écoute l'herbe. Aniss ouvre la bouche, puis la referme. Victorino tient le filet, sans le secouer. Je peux être silencieux ! Moi aussi, j'écoute. Un criquet reprend, tout près. Vous avez demandé, et ça tient. Mon chut a tenu vos pieds.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -3521,14 +3521,14 @@
       <c r="AW14" t="inlineStr">
         <is>
           <t>enfant-m|Maman, tu restes avec nous ?
-maman|Un, deux, trois, on ne bouge plus.
-narrateur|Aniss s'arrête seulement quand elle dit trois.
-narrateur|Victorino lève le filet à chaque chiffre.
-copain|Je peux attendre le trois !
-enfant-m|Moi aussi, j'attends.
-narrateur|L'herbe redevient droite, autour.
-papa|Vous avez demandé, et ça marche.
-maman|Mes chiffres ont tenu l'élan.</t>
+maman|Chut, on écoute l'herbe.
+narrateur|Aniss ouvre la bouche, puis la referme.
+narrateur|Victorino tient le filet, sans le secouer.
+copain|Je peux être silencieux !
+enfant-m|Moi aussi, j'écoute.
+narrateur|Un criquet reprend, tout près.
+papa|Vous avez demandé, et ça tient.
+maman|Mon chut a tenu vos pieds.</t>
         </is>
       </c>
     </row>
@@ -3555,12 +3555,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Le trois de maman reste dans l'air, tout léger. J'ai attendu le chiffre. On a demandé, et ça allait. Mes mots ont tenu vos pieds. Le pré vous rend le silence. Le filet vert pose un grain de jaune sur le bois. Victorino touche la tige, du bout. Il s'est posé. Une ombre de peuplier barre encore l'herbe.</t>
+          <t>Le chut de maman reste dans l'air, tout léger. J'ai fermé la bouche. On a demandé, et ça tenait. Mon silence a tenu vos pieds. Le criquet a repris, pour vous. Le filet vert pose un grain de jaune sur le bois. Victorino touche la tige, du bout. Il s'est posé. Une ombre de peuplier barre encore l'herbe.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Le trois de maman reste dans l'air, tout léger. J'ai attendu le chiffre. On a demandé, et ça allait. Mes mots ont tenu vos pieds. Le pré vous rend le silence. Le filet vert pose un grain de jaune sur le bois. Victorino touche la tige, du bout. Il s'est posé. Une ombre de peuplier barre encore l'herbe.</t>
+          <t>Le chut de maman reste dans l'air, tout léger. J'ai fermé la bouche. On a demandé, et ça tenait. Mon silence a tenu vos pieds. Le criquet a repris, pour vous. Le filet vert pose un grain de jaune sur le bois. Victorino touche la tige, du bout. Il s'est posé. Une ombre de peuplier barre encore l'herbe.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -3695,11 +3695,11 @@
       <c r="AV15" s="2" t="inlineStr"/>
       <c r="AW15" t="inlineStr">
         <is>
-          <t>narrateur|Le trois de maman reste dans l'air, tout léger.
-copain|J'ai attendu le chiffre.
-enfant-m|On a demandé, et ça allait.
-maman|Mes mots ont tenu vos pieds.
-papa|Le pré vous rend le silence.
+          <t>narrateur|Le chut de maman reste dans l'air, tout léger.
+copain|J'ai fermé la bouche.
+enfant-m|On a demandé, et ça tenait.
+maman|Mon silence a tenu vos pieds.
+papa|Le criquet a repris, pour vous.
 narrateur|Le filet vert pose un grain de jaune sur le bois.
 narrateur|Victorino touche la tige, du bout.
 copain|Il s'est posé.
@@ -3730,12 +3730,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Victorino glisse le filet entre les tiges. Les lavandes sentent partout, Aniss. Je vais jusqu'au bout, trop vite ! Ses pieds tapent les tiges, puis reviennent. La poussière violette emplit les mailles. Un parfum lève, puis retombe. Il a de l'élan, comme un petit vent. Toi tu vas plus loin, lui plus vite. On peut guetter avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Victorino glisse le filet entre les tiges. Ça sent le savon et le miel, Aniss. Je pousse les tiges, trop fort ! Un nuage de parfum saute, puis retombe. La poussière violette emplit les mailles. Le jaune quitte le violet, d'un coup. Tes pieds ont réveillé les fleurs. On s'approche sans les bousculer. Il peut revenir ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Victorino glisse le filet entre les tiges. Les lavandes sentent partout, Aniss. Je vais jusqu'au bout, trop vite ! Ses pieds tapent les tiges, puis reviennent. La poussière violette emplit les mailles. Un parfum lève, puis retombe. Il a de l'élan, comme un petit vent. Toi tu vas plus loin, lui plus vite. On peut guetter avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Victorino glisse le filet entre les tiges. Ça sent le savon et le miel, Aniss. Je pousse les tiges, trop fort ! Un nuage de parfum saute, puis retombe. La poussière violette emplit les mailles. Le jaune quitte le violet, d'un coup. Tes pieds ont réveillé les fleurs. On s'approche sans les bousculer. Il peut revenir ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -3871,14 +3871,14 @@
       <c r="AW16" t="inlineStr">
         <is>
           <t>narrateur|Victorino glisse le filet entre les tiges.
-enfant-m|Les lavandes sentent partout, Aniss.
-copain|Je vais jusqu'au bout, trop vite !
-narrateur|Ses pieds tapent les tiges, puis reviennent.
+enfant-m|Ça sent le savon et le miel, Aniss.
+copain|Je pousse les tiges, trop fort !
+narrateur|Un nuage de parfum saute, puis retombe.
 narrateur|La poussière violette emplit les mailles.
-narrateur|Un parfum lève, puis retombe.
-maman|Il a de l'élan, comme un petit vent.
-papa|Toi tu vas plus loin, lui plus vite.
-enfant-m|On peut guetter avec lui ?
+narrateur|Le jaune quitte le violet, d'un coup.
+maman|Tes pieds ont réveillé les fleurs.
+papa|On s'approche sans les bousculer.
+enfant-m|Il peut revenir ?
 papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
@@ -3911,12 +3911,12 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Les lavandes bougent encore, un peu. Souffler, attendre, ou la fleur de papa ?</t>
+          <t>Le parfum tient encore, tout bas. Souffler, attendre, ou la fleur de papa ?</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Les lavandes bougent encore, un peu. Souffler, attendre, ou la fleur de papa ?</t>
+          <t>Le parfum tient encore, tout bas. Souffler, attendre, ou la fleur de papa ?</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -4075,7 +4075,7 @@
       <c r="AV17" s="2" t="inlineStr"/>
       <c r="AW17" t="inlineStr">
         <is>
-          <t>narrateur|Les lavandes bougent encore, un peu.
+          <t>narrateur|Le parfum tient encore, tout bas.
 maman|Souffler, attendre, ou la fleur de papa ?</t>
         </is>
       </c>
@@ -4103,12 +4103,12 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>On souffle tout doux. Toi derrière, moi devant ! Victorino garde le filet, Aniss souffle devant. Deux souffles passent sur la même tige. Aniss va plus vite, Victorino plus loin. On arrive au violet, tous les deux. J'ai attendu ton souffle, un peu. Vous avez joué avec l'élan. Les lavandes vous ont laissés passer.</t>
+          <t>On souffle tout doux. Comme le petit vent ! Victorino garde le filet, Aniss souffle devant. Deux souffles passent sur la même tige. Le violet penche, puis se redresse. On n'a rien cassé. J'ai soufflé plus bas, cette fois. Vous avez joué avec l'air. Les fleurs sont restées debout.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>On souffle tout doux. Toi derrière, moi devant ! Victorino garde le filet, Aniss souffle devant. Deux souffles passent sur la même tige. Aniss va plus vite, Victorino plus loin. On arrive au violet, tous les deux. J'ai attendu ton souffle, un peu. Vous avez joué avec l'élan. Les lavandes vous ont laissés passer.</t>
+          <t>On souffle tout doux. Comme le petit vent ! Victorino garde le filet, Aniss souffle devant. Deux souffles passent sur la même tige. Le violet penche, puis se redresse. On n'a rien cassé. J'ai soufflé plus bas, cette fois. Vous avez joué avec l'air. Les fleurs sont restées debout.</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -4244,14 +4244,14 @@
       <c r="AW18" t="inlineStr">
         <is>
           <t>enfant-m|On souffle tout doux.
-copain|Toi derrière, moi devant !
+copain|Comme le petit vent !
 narrateur|Victorino garde le filet, Aniss souffle devant.
 narrateur|Deux souffles passent sur la même tige.
-narrateur|Aniss va plus vite, Victorino plus loin.
-enfant-m|On arrive au violet, tous les deux.
-copain|J'ai attendu ton souffle, un peu.
-papa|Vous avez joué avec l'élan.
-maman|Les lavandes vous ont laissés passer.</t>
+narrateur|Le violet penche, puis se redresse.
+enfant-m|On n'a rien cassé.
+copain|J'ai soufflé plus bas, cette fois.
+papa|Vous avez joué avec l'air.
+maman|Les fleurs sont restées debout.</t>
         </is>
       </c>
     </row>
@@ -4278,12 +4278,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Deux souffles marquent la même tige violette. Toi devant, moi derrière. Tes pas allaient plus loin. Vous avez soufflé avec l'élan, pas contre. Les lavandes redeviennent tièdes, et calmes. Le filet vert rentre dans le sac. Un brin violet sèche déjà sur le tissu. On rentre, le parfum reste. Le puits fait une ombre ronde.</t>
+          <t>Deux souffles marquent la même tige violette. On n'a rien cassé. J'ai soufflé plus bas. Vous avez joué avec l'air. Les lavandes sont encore debout. Le filet vert rentre dans le sac. Un brin violet sèche déjà sur le tissu. Le parfum rentre avec nous. Le puits fait une ombre ronde.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Deux souffles marquent la même tige violette. Toi devant, moi derrière. Tes pas allaient plus loin. Vous avez soufflé avec l'élan, pas contre. Les lavandes redeviennent tièdes, et calmes. Le filet vert rentre dans le sac. Un brin violet sèche déjà sur le tissu. On rentre, le parfum reste. Le puits fait une ombre ronde.</t>
+          <t>Deux souffles marquent la même tige violette. On n'a rien cassé. J'ai soufflé plus bas. Vous avez joué avec l'air. Les lavandes sont encore debout. Le filet vert rentre dans le sac. Un brin violet sèche déjà sur le tissu. Le parfum rentre avec nous. Le puits fait une ombre ronde.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -4419,13 +4419,13 @@
       <c r="AW19" t="inlineStr">
         <is>
           <t>narrateur|Deux souffles marquent la même tige violette.
-enfant-m|Toi devant, moi derrière.
-copain|Tes pas allaient plus loin.
-papa|Vous avez soufflé avec l'élan, pas contre.
-maman|Les lavandes redeviennent tièdes, et calmes.
+enfant-m|On n'a rien cassé.
+copain|J'ai soufflé plus bas.
+papa|Vous avez joué avec l'air.
+maman|Les lavandes sont encore debout.
 narrateur|Le filet vert rentre dans le sac.
 narrateur|Un brin violet sèche déjà sur le tissu.
-enfant-m|On rentre, le parfum reste.
+enfant-m|Le parfum rentre avec nous.
 narrateur|Le puits fait une ombre ronde.</t>
         </is>
       </c>
@@ -4453,12 +4453,12 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>J'attends le parfum. Moi je finis, puis c'est toi. Victorino tient le filet, sans le bouger. Aniss tapote une tige, tout seul d'abord. Il souffle, puis il recule. C'est à toi, Victorino. Merci, j'y vais. Chacun son tour, entre les tiges. L'élan a attendu le parfum.</t>
+          <t>J'attends le parfum. Quand il retombe, on avance. Victorino tient le filet, sans le bouger. Aniss compte les tiges, tout bas. Le nuage violet s'assoit, enfin. C'est à toi, Victorino. Merci, j'y vais. Le parfum vous a fait de la place. Vous l'avez laissé se poser.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>J'attends le parfum. Moi je finis, puis c'est toi. Victorino tient le filet, sans le bouger. Aniss tapote une tige, tout seul d'abord. Il souffle, puis il recule. C'est à toi, Victorino. Merci, j'y vais. Chacun son tour, entre les tiges. L'élan a attendu le parfum.</t>
+          <t>J'attends le parfum. Quand il retombe, on avance. Victorino tient le filet, sans le bouger. Aniss compte les tiges, tout bas. Le nuage violet s'assoit, enfin. C'est à toi, Victorino. Merci, j'y vais. Le parfum vous a fait de la place. Vous l'avez laissé se poser.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -4594,14 +4594,14 @@
       <c r="AW20" t="inlineStr">
         <is>
           <t>enfant-m|J'attends le parfum.
-copain|Moi je finis, puis c'est toi.
+copain|Quand il retombe, on avance.
 narrateur|Victorino tient le filet, sans le bouger.
-narrateur|Aniss tapote une tige, tout seul d'abord.
-narrateur|Il souffle, puis il recule.
+narrateur|Aniss compte les tiges, tout bas.
+narrateur|Le nuage violet s'assoit, enfin.
 copain|C'est à toi, Victorino.
 enfant-m|Merci, j'y vais.
-papa|Chacun son tour, entre les tiges.
-maman|L'élan a attendu le parfum.</t>
+papa|Le parfum vous a fait de la place.
+maman|Vous l'avez laissé se poser.</t>
         </is>
       </c>
     </row>
@@ -4628,12 +4628,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Le parfum attend encore, tout bas. J'ai fini, puis c'était toi. J'ai attendu ta tige. Chacun son tour, entre les tiges. L'élan a laissé la place. Le filet vert garde un grain de parfum. Victorino souffle dessus, tout doux. On se dit au revoir, lavandes. Une abeille passe, sans se presser.</t>
+          <t>Le parfum s'est assis, tout bas. Quand il est retombé, on a avancé. J'ai attendu ta tige. Le nuage vous a laissés passer. Vous l'avez laissé se poser. Le filet vert garde un grain de parfum. Victorino souffle dessus, tout doux. Au revoir, les tiges. Une abeille passe, sans se presser.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Le parfum attend encore, tout bas. J'ai fini, puis c'était toi. J'ai attendu ta tige. Chacun son tour, entre les tiges. L'élan a laissé la place. Le filet vert garde un grain de parfum. Victorino souffle dessus, tout doux. On se dit au revoir, lavandes. Une abeille passe, sans se presser.</t>
+          <t>Le parfum s'est assis, tout bas. Quand il est retombé, on a avancé. J'ai attendu ta tige. Le nuage vous a laissés passer. Vous l'avez laissé se poser. Le filet vert garde un grain de parfum. Victorino souffle dessus, tout doux. Au revoir, les tiges. Une abeille passe, sans se presser.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -4768,14 +4768,14 @@
       <c r="AV21" s="2" t="inlineStr"/>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>narrateur|Le parfum attend encore, tout bas.
-copain|J'ai fini, puis c'était toi.
+          <t>narrateur|Le parfum s'est assis, tout bas.
+copain|Quand il est retombé, on a avancé.
 enfant-m|J'ai attendu ta tige.
-maman|Chacun son tour, entre les tiges.
-papa|L'élan a laissé la place.
+maman|Le nuage vous a laissés passer.
+papa|Vous l'avez laissé se poser.
 narrateur|Le filet vert garde un grain de parfum.
 narrateur|Victorino souffle dessus, tout doux.
-copain|On se dit au revoir, lavandes.
+copain|Au revoir, les tiges.
 narrateur|Une abeille passe, sans se presser.</t>
         </is>
       </c>
@@ -4803,12 +4803,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu gardes la fleur ? Je la tends, un pas chacun. Papa pose la fleur près du filet. Aniss s'approche, tout petit pas. Victorino s'approche, encore plus lent. On demande, et ça va ! Le violet est à nous. Vous avez demandé, tout calme. Ma main a juste attendu.</t>
+          <t>Papa, tu gardes la fleur ? Je la tends, un pas chacun. Papa pose la fleur près du filet. Aniss pose un pied, puis l'autre. Victorino pose le même pas, plus tard. On a demandé, et ça va ! Le violet est tout près. Vous avez demandé, tout calme. Ma main n'a pas bougé.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu gardes la fleur ? Je la tends, un pas chacun. Papa pose la fleur près du filet. Aniss s'approche, tout petit pas. Victorino s'approche, encore plus lent. On demande, et ça va ! Le violet est à nous. Vous avez demandé, tout calme. Ma main a juste attendu.</t>
+          <t>Papa, tu gardes la fleur ? Je la tends, un pas chacun. Papa pose la fleur près du filet. Aniss pose un pied, puis l'autre. Victorino pose le même pas, plus tard. On a demandé, et ça va ! Le violet est tout près. Vous avez demandé, tout calme. Ma main n'a pas bougé.</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -4946,12 +4946,12 @@
           <t>enfant-m|Papa, tu gardes la fleur ?
 papa|Je la tends, un pas chacun.
 narrateur|Papa pose la fleur près du filet.
-narrateur|Aniss s'approche, tout petit pas.
-narrateur|Victorino s'approche, encore plus lent.
-copain|On demande, et ça va !
-enfant-m|Le violet est à nous.
+narrateur|Aniss pose un pied, puis l'autre.
+narrateur|Victorino pose le même pas, plus tard.
+copain|On a demandé, et ça va !
+enfant-m|Le violet est tout près.
 maman|Vous avez demandé, tout calme.
-papa|Ma main a juste attendu.</t>
+papa|Ma main n'a pas bougé.</t>
         </is>
       </c>
     </row>
@@ -4978,12 +4978,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>La fleur de papa repose près du violet. Tu la tendais, un pas chacun. On a demandé, et ça venait juste. Ma main a fait le tour, rien de plus. Les lavandes ont rendu le jaune. Le filet vert rentre dans le sac. Un rond clair reste sur une feuille. Regarde, Aniss, il brille. Le chat reprend la pierre, au frais.</t>
+          <t>La fleur de papa repose près du violet. Tu la tendais, un pas chacun. On a demandé, et ça venait juste. Ma main n'a pas bougé. Les lavandes ont rendu le jaune. Le filet vert rentre dans le sac. Un rond clair reste sur une feuille. Regarde, Aniss, il brille. Le chat reprend la pierre, au frais.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>La fleur de papa repose près du violet. Tu la tendais, un pas chacun. On a demandé, et ça venait juste. Ma main a fait le tour, rien de plus. Les lavandes ont rendu le jaune. Le filet vert rentre dans le sac. Un rond clair reste sur une feuille. Regarde, Aniss, il brille. Le chat reprend la pierre, au frais.</t>
+          <t>La fleur de papa repose près du violet. Tu la tendais, un pas chacun. On a demandé, et ça venait juste. Ma main n'a pas bougé. Les lavandes ont rendu le jaune. Le filet vert rentre dans le sac. Un rond clair reste sur une feuille. Regarde, Aniss, il brille. Le chat reprend la pierre, au frais.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -5121,7 +5121,7 @@
           <t>narrateur|La fleur de papa repose près du violet.
 enfant-m|Tu la tendais, un pas chacun.
 copain|On a demandé, et ça venait juste.
-papa|Ma main a fait le tour, rien de plus.
+papa|Ma main n'a pas bougé.
 maman|Les lavandes ont rendu le jaune.
 narrateur|Le filet vert rentre dans le sac.
 narrateur|Un rond clair reste sur une feuille.
@@ -5153,12 +5153,12 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Victorino pose le filet contre la pierre. Ici, la pierre est chaude, Aniss. J'entends mes pieds deux fois ! Le muret renvoie chaque pas, tout fort. Les pas d'Aniss font trembler le filet. Le filet vert attend au bord, un peu seule. Son élan remplit toute la pierre. Toi tu vas plus loin, lui plus vite. On guette comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Victorino pose le filet contre la pierre. La pierre est tiède, Aniss. J'entends mes pieds deux fois ! Chaque clic revient, plus fort. Les pas d'Aniss font trembler le filet. Le filet vert n'ose plus bouger. Le jaune n'aime pas le bruit. La pierre répète tes pas. On fait moins de clic ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Victorino pose le filet contre la pierre. Ici, la pierre est chaude, Aniss. J'entends mes pieds deux fois ! Le muret renvoie chaque pas, tout fort. Les pas d'Aniss font trembler le filet. Le filet vert attend au bord, un peu seule. Son élan remplit toute la pierre. Toi tu vas plus loin, lui plus vite. On guette comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Victorino pose le filet contre la pierre. La pierre est tiède, Aniss. J'entends mes pieds deux fois ! Chaque clic revient, plus fort. Les pas d'Aniss font trembler le filet. Le filet vert n'ose plus bouger. Le jaune n'aime pas le bruit. La pierre répète tes pas. On fait moins de clic ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -5294,14 +5294,14 @@
       <c r="AW24" t="inlineStr">
         <is>
           <t>narrateur|Victorino pose le filet contre la pierre.
-enfant-m|Ici, la pierre est chaude, Aniss.
+enfant-m|La pierre est tiède, Aniss.
 copain|J'entends mes pieds deux fois !
-narrateur|Le muret renvoie chaque pas, tout fort.
+narrateur|Chaque clic revient, plus fort.
 narrateur|Les pas d'Aniss font trembler le filet.
-narrateur|Le filet vert attend au bord, un peu seule.
-maman|Son élan remplit toute la pierre.
-papa|Toi tu vas plus loin, lui plus vite.
-copain|On guette comment, alors ?
+narrateur|Le filet vert n'ose plus bouger.
+maman|Le jaune n'aime pas le bruit.
+papa|La pierre répète tes pas.
+copain|On fait moins de clic ?
 papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
@@ -5329,12 +5329,12 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Les clics remplissent encore le muret. Le rythme, en bas, ou la main de maman ?</t>
+          <t>Un dernier clic roule le long du muret. Le rythme, en bas, ou la main de maman ?</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Les clics remplissent encore le muret. Le rythme, en bas, ou la main de maman ?</t>
+          <t>Un dernier clic roule le long du muret. Le rythme, en bas, ou la main de maman ?</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -5493,7 +5493,7 @@
       <c r="AV25" s="2" t="inlineStr"/>
       <c r="AW25" t="inlineStr">
         <is>
-          <t>narrateur|Les clics remplissent encore le muret.
+          <t>narrateur|Un dernier clic roule le long du muret.
 papa|Le rythme, en bas, ou la main de maman ?</t>
         </is>
       </c>
@@ -5521,12 +5521,12 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>On fait un rythme sur la pierre. Toc toc, j'avance ! Victorino pose une main sur l'épaule d'Aniss. Le filet vert voyage contre la pierre, entre deux taps. Ils tapent la même pierre, l'un après l'autre. Doucement, le rythme tient. Le clic suit le rythme, puis se tait. Vous jouez avec le bruit, ensemble. Le muret est devenu un tambour.</t>
+          <t>On tape une fois, puis plus. Toc, et j'attends. Victorino pose une main sur l'épaule d'Aniss. Le filet vert se pose après le dernier toc. La pierre répond, puis se tait. Le jaune aime le silence, après. Moi aussi, après le toc. Vous avez joué avec le bruit. Un toc, puis la pierre dort.</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>On fait un rythme sur la pierre. Toc toc, j'avance ! Victorino pose une main sur l'épaule d'Aniss. Le filet vert voyage contre la pierre, entre deux taps. Ils tapent la même pierre, l'un après l'autre. Doucement, le rythme tient. Le clic suit le rythme, puis se tait. Vous jouez avec le bruit, ensemble. Le muret est devenu un tambour.</t>
+          <t>On tape une fois, puis plus. Toc, et j'attends. Victorino pose une main sur l'épaule d'Aniss. Le filet vert se pose après le dernier toc. La pierre répond, puis se tait. Le jaune aime le silence, après. Moi aussi, après le toc. Vous avez joué avec le bruit. Un toc, puis la pierre dort.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -5661,15 +5661,15 @@
       <c r="AV26" s="2" t="inlineStr"/>
       <c r="AW26" t="inlineStr">
         <is>
-          <t>enfant-m|On fait un rythme sur la pierre.
-copain|Toc toc, j'avance !
+          <t>enfant-m|On tape une fois, puis plus.
+copain|Toc, et j'attends.
 narrateur|Victorino pose une main sur l'épaule d'Aniss.
-narrateur|Le filet vert voyage contre la pierre, entre deux taps.
-narrateur|Ils tapent la même pierre, l'un après l'autre.
-enfant-m|Doucement, le rythme tient.
-copain|Le clic suit le rythme, puis se tait.
-papa|Vous jouez avec le bruit, ensemble.
-maman|Le muret est devenu un tambour.</t>
+narrateur|Le filet vert se pose après le dernier toc.
+narrateur|La pierre répond, puis se tait.
+enfant-m|Le jaune aime le silence, après.
+copain|Moi aussi, après le toc.
+papa|Vous avez joué avec le bruit.
+maman|Un toc, puis la pierre dort.</t>
         </is>
       </c>
     </row>
@@ -5696,12 +5696,12 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Le rythme s'arrête, et le jaune se pose. Toc toc, on est arrivés. J'avais la main sur ton épaule. Le muret est redevenu une pierre, simplement. Le clic s'est couché. Le filet vert rentre dans le sac. Une poussière tourne encore, puis tombe. On rentre, le tambour se tait. Dehors, le pré redevient calme.</t>
+          <t>Après le toc, le jaune se pose. J'ai tapé une fois, puis plus. J'avais la main sur ton épaule. La pierre a fini par dormir. Un toc, puis le silence. Le filet vert rentre dans le sac. Une poussière tourne encore, puis tombe. Le muret s'est tu. Dehors, le pré redevient calme.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Le rythme s'arrête, et le jaune se pose. Toc toc, on est arrivés. J'avais la main sur ton épaule. Le muret est redevenu une pierre, simplement. Le clic s'est couché. Le filet vert rentre dans le sac. Une poussière tourne encore, puis tombe. On rentre, le tambour se tait. Dehors, le pré redevient calme.</t>
+          <t>Après le toc, le jaune se pose. J'ai tapé une fois, puis plus. J'avais la main sur ton épaule. La pierre a fini par dormir. Un toc, puis le silence. Le filet vert rentre dans le sac. Une poussière tourne encore, puis tombe. Le muret s'est tu. Dehors, le pré redevient calme.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -5836,14 +5836,14 @@
       <c r="AV27" s="2" t="inlineStr"/>
       <c r="AW27" t="inlineStr">
         <is>
-          <t>narrateur|Le rythme s'arrête, et le jaune se pose.
-copain|Toc toc, on est arrivés.
+          <t>narrateur|Après le toc, le jaune se pose.
+copain|J'ai tapé une fois, puis plus.
 enfant-m|J'avais la main sur ton épaule.
-papa|Le muret est redevenu une pierre, simplement.
-maman|Le clic s'est couché.
+papa|La pierre a fini par dormir.
+maman|Un toc, puis le silence.
 narrateur|Le filet vert rentre dans le sac.
 narrateur|Une poussière tourne encore, puis tombe.
-enfant-m|On rentre, le tambour se tait.
+enfant-m|Le muret s'est tu.
 narrateur|Dehors, le pré redevient calme.</t>
         </is>
       </c>
@@ -5871,12 +5871,12 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>On attend en bas. Quand la pierre se tait, je m'approche. Un pas dans l'herbe, puis plus rien. Le filet vert reste muet, au creux. Le muret se tait, enfin. Maintenant ! À toi, puis à moi. Vous avez laissé le bruit s'asseoir. L'élan a attendu le silence.</t>
+          <t>On attend en bas. La pierre se tait, d'abord. Leurs chaussures restent dans l'herbe fraîche. Le filet vert reste dans l'herbe, en bas. Le muret ne clique plus. Maintenant, on peut regarder. À toi, puis à moi. Vous avez laissé le bruit s'en aller. En bas, vos pieds sont plus doux.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>On attend en bas. Quand la pierre se tait, je m'approche. Un pas dans l'herbe, puis plus rien. Le filet vert reste muet, au creux. Le muret se tait, enfin. Maintenant ! À toi, puis à moi. Vous avez laissé le bruit s'asseoir. L'élan a attendu le silence.</t>
+          <t>On attend en bas. La pierre se tait, d'abord. Leurs chaussures restent dans l'herbe fraîche. Le filet vert reste dans l'herbe, en bas. Le muret ne clique plus. Maintenant, on peut regarder. À toi, puis à moi. Vous avez laissé le bruit s'en aller. En bas, vos pieds sont plus doux.</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -6012,14 +6012,14 @@
       <c r="AW28" t="inlineStr">
         <is>
           <t>enfant-m|On attend en bas.
-copain|Quand la pierre se tait, je m'approche.
-narrateur|Un pas dans l'herbe, puis plus rien.
-narrateur|Le filet vert reste muet, au creux.
-narrateur|Le muret se tait, enfin.
-copain|Maintenant !
+copain|La pierre se tait, d'abord.
+narrateur|Leurs chaussures restent dans l'herbe fraîche.
+narrateur|Le filet vert reste dans l'herbe, en bas.
+narrateur|Le muret ne clique plus.
+copain|Maintenant, on peut regarder.
 enfant-m|À toi, puis à moi.
-papa|Vous avez laissé le bruit s'asseoir.
-maman|L'élan a attendu le silence.</t>
+papa|Vous avez laissé le bruit s'en aller.
+maman|En bas, vos pieds sont plus doux.</t>
         </is>
       </c>
     </row>
@@ -6046,12 +6046,12 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>La pierre s'est tue, enfin, tout à fait. On a attendu en bas. Quand elle était partie, on s'approchait. Le silence vous a laissé le jaune. L'élan a écouté la pierre. Le filet vert ne fait plus aucun bruit. Victorino pose la paume sur la pierre chaude. Elle est tiède. Un oiseau passe au-dessus du muret, sans crier.</t>
+          <t>La pierre s'est tue, enfin, tout à fait. On a attendu en bas. Nos chaussures sont restées dans l'herbe. Le silence vous a laissé le jaune. En bas, vos pieds étaient plus doux. Le filet vert ne fait plus aucun bruit. Victorino pose la paume sur la pierre chaude. Elle est tiède. Un oiseau passe au-dessus du muret, sans crier.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>La pierre s'est tue, enfin, tout à fait. On a attendu en bas. Quand elle était partie, on s'approchait. Le silence vous a laissé le jaune. L'élan a écouté la pierre. Le filet vert ne fait plus aucun bruit. Victorino pose la paume sur la pierre chaude. Elle est tiède. Un oiseau passe au-dessus du muret, sans crier.</t>
+          <t>La pierre s'est tue, enfin, tout à fait. On a attendu en bas. Nos chaussures sont restées dans l'herbe. Le silence vous a laissé le jaune. En bas, vos pieds étaient plus doux. Le filet vert ne fait plus aucun bruit. Victorino pose la paume sur la pierre chaude. Elle est tiède. Un oiseau passe au-dessus du muret, sans crier.</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -6188,9 +6188,9 @@
         <is>
           <t>narrateur|La pierre s'est tue, enfin, tout à fait.
 enfant-m|On a attendu en bas.
-copain|Quand elle était partie, on s'approchait.
+copain|Nos chaussures sont restées dans l'herbe.
 papa|Le silence vous a laissé le jaune.
-maman|L'élan a écouté la pierre.
+maman|En bas, vos pieds étaient plus doux.
 narrateur|Le filet vert ne fait plus aucun bruit.
 narrateur|Victorino pose la paume sur la pierre chaude.
 copain|Elle est tiède.
@@ -6221,12 +6221,12 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tends la main ? Je reste, et vous venez tout doux. Aniss écoute la paume, plus que ses pieds. Victorino lève le filet quand maman ouvre la paume. Je m'arrête sur ta main ! Moi aussi, j'écoute. Le clic se range derrière le silence. Vous avez demandé la main. Ma paume a tenu l'élan.</t>
+          <t>Maman, tu tends la main ? Je reste, et vous venez tout doux. Aniss regarde la paume, plus que ses pieds. Victorino lève le filet quand maman ouvre la paume. Je m'arrête devant ta main ! Moi aussi, j'écoute. Un grain de foin dort dans ses plis. Vous avez demandé la main. Ma paume est devenue une tige.</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tends la main ? Je reste, et vous venez tout doux. Aniss écoute la paume, plus que ses pieds. Victorino lève le filet quand maman ouvre la paume. Je m'arrête sur ta main ! Moi aussi, j'écoute. Le clic se range derrière le silence. Vous avez demandé la main. Ma paume a tenu l'élan.</t>
+          <t>Maman, tu tends la main ? Je reste, et vous venez tout doux. Aniss regarde la paume, plus que ses pieds. Victorino lève le filet quand maman ouvre la paume. Je m'arrête devant ta main ! Moi aussi, j'écoute. Un grain de foin dort dans ses plis. Vous avez demandé la main. Ma paume est devenue une tige.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -6363,13 +6363,13 @@
         <is>
           <t>enfant-m|Maman, tu tends la main ?
 maman|Je reste, et vous venez tout doux.
-narrateur|Aniss écoute la paume, plus que ses pieds.
+narrateur|Aniss regarde la paume, plus que ses pieds.
 narrateur|Victorino lève le filet quand maman ouvre la paume.
-copain|Je m'arrête sur ta main !
+copain|Je m'arrête devant ta main !
 enfant-m|Moi aussi, j'écoute.
-narrateur|Le clic se range derrière le silence.
+narrateur|Un grain de foin dort dans ses plis.
 papa|Vous avez demandé la main.
-maman|Ma paume a tenu l'élan.</t>
+maman|Ma paume est devenue une tige.</t>
         </is>
       </c>
     </row>
@@ -6396,12 +6396,12 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>La paume de maman s'ouvre, puis se referme. J'écoutais ta main. Moi aussi, je m'arrêtais dessus. Vous avez demandé le calme. Le muret a rendu vos pas. Le filet vert rentre dans le sac. Victorino touche la pierre, du bout des doigts. Il s'est posé, Aniss. La pierre garde une poussière, puis plus rien.</t>
+          <t>La paume de maman s'ouvre, puis se referme. J'écoutais ta main. Moi aussi, je m'arrêtais dessus. Vous avez demandé le calme. Un grain de foin reste dans ses plis. Le filet vert rentre dans le sac. Victorino touche la pierre, du bout des doigts. Il s'est posé, Aniss. La pierre garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>La paume de maman s'ouvre, puis se referme. J'écoutais ta main. Moi aussi, je m'arrêtais dessus. Vous avez demandé le calme. Le muret a rendu vos pas. Le filet vert rentre dans le sac. Victorino touche la pierre, du bout des doigts. Il s'est posé, Aniss. La pierre garde une poussière, puis plus rien.</t>
+          <t>La paume de maman s'ouvre, puis se referme. J'écoutais ta main. Moi aussi, je m'arrêtais dessus. Vous avez demandé le calme. Un grain de foin reste dans ses plis. Le filet vert rentre dans le sac. Victorino touche la pierre, du bout des doigts. Il s'est posé, Aniss. La pierre garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -6540,7 +6540,7 @@
 enfant-m|J'écoutais ta main.
 copain|Moi aussi, je m'arrêtais dessus.
 maman|Vous avez demandé le calme.
-papa|Le muret a rendu vos pas.
+papa|Un grain de foin reste dans ses plis.
 narrateur|Le filet vert rentre dans le sac.
 narrateur|Victorino touche la pierre, du bout des doigts.
 enfant-m|Il s'est posé, Aniss.
@@ -6933,12 +6933,12 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Le chapeau veille déjà sur les sourcils. Je vois l'ombre ! Ne cours pas encore. Aniss a les cheveux tout courts. Une mèche saute quand il respire. Ça sent déjà le foin, derrière le portail. Vos mains, au-dessus du sac ? Oui, maman.</t>
+          <t>Le bord du chapeau coupe le soleil. Je suis tout petit, dessous ! Reste près de moi, d'abord. Aniss cligne, trop vite. Une mèche lui saute sur l'œil. Le foin sent déjà, dehors. Le sac est fermé ? Oui, maman.</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Le chapeau veille déjà sur les sourcils. Je vois l'ombre ! Ne cours pas encore. Aniss a les cheveux tout courts. Une mèche saute quand il respire. Ça sent déjà le foin, derrière le portail. Vos mains, au-dessus du sac ? Oui, maman.</t>
+          <t>Le bord du chapeau coupe le soleil. Je suis tout petit, dessous ! Reste près de moi, d'abord. Aniss cligne, trop vite. Une mèche lui saute sur l'œil. Le foin sent déjà, dehors. Le sac est fermé ? Oui, maman.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -7077,13 +7077,13 @@
       </c>
       <c r="AW34" t="inlineStr">
         <is>
-          <t>narrateur|Le chapeau veille déjà sur les sourcils.
-copain|Je vois l'ombre !
-enfant-m|Ne cours pas encore.
-narrateur|Aniss a les cheveux tout courts.
-narrateur|Une mèche saute quand il respire.
-papa|Ça sent déjà le foin, derrière le portail.
-maman|Vos mains, au-dessus du sac ?
+          <t>narrateur|Le bord du chapeau coupe le soleil.
+copain|Je suis tout petit, dessous !
+enfant-m|Reste près de moi, d'abord.
+narrateur|Aniss cligne, trop vite.
+narrateur|Une mèche lui saute sur l'œil.
+papa|Le foin sent déjà, dehors.
+maman|Le sac est fermé ?
 copain|Oui, maman.</t>
         </is>
       </c>
@@ -7111,12 +7111,12 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Aniss tapote déjà le sol, tout léger. Le pré a l'herbe haute, encore tiède. Les lavandes sentent fort, tout bas. Le muret garde une pierre chaude. On commence où, pour le papillon ?</t>
+          <t>Aniss tape déjà deux cailloux, l'un contre l'autre. Le pré ondule, plus loin que le puits. Les lavandes font un mur violet, tout bas. Le muret tient encore la chaleur du chat. On guette où, d'abord ?</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Aniss tapote déjà le sol, tout léger. Le pré a l'herbe haute, encore tiède. Les lavandes sentent fort, tout bas. Le muret garde une pierre chaude. On commence où, pour le papillon ?</t>
+          <t>Aniss tape déjà deux cailloux, l'un contre l'autre. Le pré ondule, plus loin que le puits. Les lavandes font un mur violet, tout bas. Le muret tient encore la chaleur du chat. On guette où, d'abord ?</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -7275,11 +7275,11 @@
       <c r="AV35" s="2" t="inlineStr"/>
       <c r="AW35" t="inlineStr">
         <is>
-          <t>narrateur|Aniss tapote déjà le sol, tout léger.
-narrateur|Le pré a l'herbe haute, encore tiède.
-narrateur|Les lavandes sentent fort, tout bas.
-narrateur|Le muret garde une pierre chaude.
-papa|On commence où, pour le papillon ?</t>
+          <t>narrateur|Aniss tape déjà deux cailloux, l'un contre l'autre.
+narrateur|Le pré ondule, plus loin que le puits.
+narrateur|Les lavandes font un mur violet, tout bas.
+narrateur|Le muret tient encore la chaleur du chat.
+papa|On guette où, d'abord ?</t>
         </is>
       </c>
     </row>
@@ -7306,12 +7306,12 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Victorino baisse le chapeau, pour l'ombre. L'herbe du pré sent le foin chaud. Moi je cours, Victorino ! Aniss fend l'herbe, trop vite. Un nuage de graines s'envole, tout haut. Le chapeau s'envole, puis retombe. Le chapeau bleu n'attendait pas ça. Il a envie de bouger, c'est tout. Ses jambes sont plus courtes, plus vives. On guette comment, alors ? Vous faites comment, tous les deux ?</t>
+          <t>Victorino baisse le chapeau, pour l'ombre. Les tiges se touchent, puis se séparent. Je le rattrape ! Aniss part dans l'herbe, trop loin. Le jaune s'envole, plus haut que leurs têtes. Le chapeau s'envole, puis retombe. Le chapeau bleu n'a pas suffi. Il a envie de courir, c'est tout. Tes pieds vont trop vite, Aniss. Je fais comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Victorino baisse le chapeau, pour l'ombre. L'herbe du pré sent le foin chaud. Moi je cours, Victorino ! Aniss fend l'herbe, trop vite. Un nuage de graines s'envole, tout haut. Le chapeau s'envole, puis retombe. Le chapeau bleu n'attendait pas ça. Il a envie de bouger, c'est tout. Ses jambes sont plus courtes, plus vives. On guette comment, alors ? Vous faites comment, tous les deux ?</t>
+          <t>Victorino baisse le chapeau, pour l'ombre. Les tiges se touchent, puis se séparent. Je le rattrape ! Aniss part dans l'herbe, trop loin. Le jaune s'envole, plus haut que leurs têtes. Le chapeau s'envole, puis retombe. Le chapeau bleu n'a pas suffi. Il a envie de courir, c'est tout. Tes pieds vont trop vite, Aniss. Je fais comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -7447,16 +7447,16 @@
       <c r="AW36" t="inlineStr">
         <is>
           <t>narrateur|Victorino baisse le chapeau, pour l'ombre.
-narrateur|L'herbe du pré sent le foin chaud.
-copain|Moi je cours, Victorino !
-narrateur|Aniss fend l'herbe, trop vite.
-narrateur|Un nuage de graines s'envole, tout haut.
+narrateur|Les tiges se touchent, puis se séparent.
+copain|Je le rattrape !
+narrateur|Aniss part dans l'herbe, trop loin.
+narrateur|Le jaune s'envole, plus haut que leurs têtes.
 narrateur|Le chapeau s'envole, puis retombe.
-enfant-m|Le chapeau bleu n'attendait pas ça.
-maman|Il a envie de bouger, c'est tout.
-papa|Ses jambes sont plus courtes, plus vives.
-copain|On guette comment, alors ?
-papa|Vous faites comment, tous les deux ?</t>
+enfant-m|Le chapeau bleu n'a pas suffi.
+maman|Il a envie de courir, c'est tout.
+papa|Tes pieds vont trop vite, Aniss.
+copain|Je fais comment, alors ?
+papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="AX36" t="inlineStr">
@@ -7488,12 +7488,12 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Aniss fend encore l'herbe, tout léger. Marcher comme lui, s'asseoir, ou maman ?</t>
+          <t>L'herbe se referme derrière Aniss. Marcher comme lui, s'asseoir, ou le silence ?</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Aniss fend encore l'herbe, tout léger. Marcher comme lui, s'asseoir, ou maman ?</t>
+          <t>L'herbe se referme derrière Aniss. Marcher comme lui, s'asseoir, ou le silence ?</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -7652,8 +7652,8 @@
       <c r="AV37" s="2" t="inlineStr"/>
       <c r="AW37" t="inlineStr">
         <is>
-          <t>narrateur|Aniss fend encore l'herbe, tout léger.
-papa|Marcher comme lui, s'asseoir, ou maman ?</t>
+          <t>narrateur|L'herbe se referme derrière Aniss.
+papa|Marcher comme lui, s'asseoir, ou le silence ?</t>
         </is>
       </c>
     </row>
@@ -7680,12 +7680,12 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>On marche comme lui. Moi je bats des bras, tout lent. Aniss tient le sac, Victorino baisse le chapeau. Deux ombres avancent dans l'herbe, sans courir. Aniss lève un pied, puis s'arrête. Maintenant c'est moi. Puis c'est moi encore. Vous jouez à son pas. L'élan a trouvé sa place.</t>
+          <t>On marche comme lui. Moi je bats des bras, tout lent. Le chapeau fait une ombre, tout lente. Deux ombres avancent dans l'herbe, sans courir. Aniss lève un pied, puis le repose. Le jaune a des ailes comme ça. Les miennes aussi, maintenant. Vous jouez à son pas. Le pré vous a laissés entrer.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>On marche comme lui. Moi je bats des bras, tout lent. Aniss tient le sac, Victorino baisse le chapeau. Deux ombres avancent dans l'herbe, sans courir. Aniss lève un pied, puis s'arrête. Maintenant c'est moi. Puis c'est moi encore. Vous jouez à son pas. L'élan a trouvé sa place.</t>
+          <t>On marche comme lui. Moi je bats des bras, tout lent. Le chapeau fait une ombre, tout lente. Deux ombres avancent dans l'herbe, sans courir. Aniss lève un pied, puis le repose. Le jaune a des ailes comme ça. Les miennes aussi, maintenant. Vous jouez à son pas. Le pré vous a laissés entrer.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -7822,13 +7822,13 @@
         <is>
           <t>enfant-m|On marche comme lui.
 copain|Moi je bats des bras, tout lent.
-narrateur|Aniss tient le sac, Victorino baisse le chapeau.
+narrateur|Le chapeau fait une ombre, tout lente.
 narrateur|Deux ombres avancent dans l'herbe, sans courir.
-narrateur|Aniss lève un pied, puis s'arrête.
-enfant-m|Maintenant c'est moi.
-copain|Puis c'est moi encore.
+narrateur|Aniss lève un pied, puis le repose.
+enfant-m|Le jaune a des ailes comme ça.
+copain|Les miennes aussi, maintenant.
 papa|Vous jouez à son pas.
-maman|L'élan a trouvé sa place.</t>
+maman|Le pré vous a laissés entrer.</t>
         </is>
       </c>
     </row>
@@ -7855,12 +7855,12 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Le papillon jaune se pose, au bout d'une tige. On a marché, chacun son tour. Tu battais des bras, moi j'avançais. Vous avez laissé l'élan dessiner. Le pré sent encore le foin. Le chapeau bleu reste sur les cheveux. Une poudre jaune dort sur l'herbe. On rentre, Aniss. Le portail de bois cliquette, tout seul.</t>
+          <t>Le papillon jaune se pose, au bout d'une tige. Mes bras ont fait des ailes. Les miennes aussi, tout lent. Vous avez marché à son pas. Le pré sent encore le foin. Le chapeau bleu reste sur les cheveux. Une poudre jaune dort sur l'herbe. Il est venu, Aniss. Le portail de bois cliquette, tout seul.</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Le papillon jaune se pose, au bout d'une tige. On a marché, chacun son tour. Tu battais des bras, moi j'avançais. Vous avez laissé l'élan dessiner. Le pré sent encore le foin. Le chapeau bleu reste sur les cheveux. Une poudre jaune dort sur l'herbe. On rentre, Aniss. Le portail de bois cliquette, tout seul.</t>
+          <t>Le papillon jaune se pose, au bout d'une tige. Mes bras ont fait des ailes. Les miennes aussi, tout lent. Vous avez marché à son pas. Le pré sent encore le foin. Le chapeau bleu reste sur les cheveux. Une poudre jaune dort sur l'herbe. Il est venu, Aniss. Le portail de bois cliquette, tout seul.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -7996,13 +7996,13 @@
       <c r="AW39" t="inlineStr">
         <is>
           <t>narrateur|Le papillon jaune se pose, au bout d'une tige.
-copain|On a marché, chacun son tour.
-enfant-m|Tu battais des bras, moi j'avançais.
-papa|Vous avez laissé l'élan dessiner.
+copain|Mes bras ont fait des ailes.
+enfant-m|Les miennes aussi, tout lent.
+papa|Vous avez marché à son pas.
 maman|Le pré sent encore le foin.
 narrateur|Le chapeau bleu reste sur les cheveux.
 narrateur|Une poudre jaune dort sur l'herbe.
-enfant-m|On rentre, Aniss.
+enfant-m|Il est venu, Aniss.
 narrateur|Le portail de bois cliquette, tout seul.</t>
         </is>
       </c>
@@ -8030,12 +8030,12 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>On s'assoit un peu. Je m'assois, alors. Aniss pose les genoux dans l'herbe. Le chapeau bleu attend près des genoux. Sa respiration redevient calme, tout doux. Tu es prêt ? Je ne cours plus. Vous avez laissé l'élan s'asseoir. Le pré vous a gardés.</t>
+          <t>On s'assoit un peu. Je m'assois, alors. Aniss pose les genoux dans l'herbe. Le chapeau bleu fait un toit, assis. Une tige se redresse, tout contre sa chaussure. Tu es prêt ? Je ne cours plus. Vous avez attendu l'herbe. Le jaune peut redescendre, maintenant.</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>On s'assoit un peu. Je m'assois, alors. Aniss pose les genoux dans l'herbe. Le chapeau bleu attend près des genoux. Sa respiration redevient calme, tout doux. Tu es prêt ? Je ne cours plus. Vous avez laissé l'élan s'asseoir. Le pré vous a gardés.</t>
+          <t>On s'assoit un peu. Je m'assois, alors. Aniss pose les genoux dans l'herbe. Le chapeau bleu fait un toit, assis. Une tige se redresse, tout contre sa chaussure. Tu es prêt ? Je ne cours plus. Vous avez attendu l'herbe. Le jaune peut redescendre, maintenant.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -8173,12 +8173,12 @@
           <t>enfant-m|On s'assoit un peu.
 copain|Je m'assois, alors.
 narrateur|Aniss pose les genoux dans l'herbe.
-narrateur|Le chapeau bleu attend près des genoux.
-narrateur|Sa respiration redevient calme, tout doux.
+narrateur|Le chapeau bleu fait un toit, assis.
+narrateur|Une tige se redresse, tout contre sa chaussure.
 enfant-m|Tu es prêt ?
 copain|Je ne cours plus.
-papa|Vous avez laissé l'élan s'asseoir.
-maman|Le pré vous a gardés.</t>
+papa|Vous avez attendu l'herbe.
+maman|Le jaune peut redescendre, maintenant.</t>
         </is>
       </c>
     </row>
@@ -8205,12 +8205,12 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>L'herbe garde encore la chaleur des genoux. Tu t'es assis, d'abord. Puis le jaune est venu, tout droit. L'élan s'est assis, puis il a guetté. Le pré redevient calme. Le chapeau bleu reste sur les cheveux. Une graine reste coincée au tissu. À demain, les tiges. Le gravier du chemin brille un peu.</t>
+          <t>L'herbe garde encore la chaleur des genoux. Tu t'es assis, d'abord. Puis le jaune est venu, tout droit. Vous avez attendu, assis. Une tige vous a chatouillés, sans rien dire. Le chapeau bleu reste sur les cheveux. Une graine reste coincée au tissu. À demain, les tiges. Le gravier du chemin brille un peu.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>L'herbe garde encore la chaleur des genoux. Tu t'es assis, d'abord. Puis le jaune est venu, tout droit. L'élan s'est assis, puis il a guetté. Le pré redevient calme. Le chapeau bleu reste sur les cheveux. Une graine reste coincée au tissu. À demain, les tiges. Le gravier du chemin brille un peu.</t>
+          <t>L'herbe garde encore la chaleur des genoux. Tu t'es assis, d'abord. Puis le jaune est venu, tout droit. Vous avez attendu, assis. Une tige vous a chatouillés, sans rien dire. Le chapeau bleu reste sur les cheveux. Une graine reste coincée au tissu. À demain, les tiges. Le gravier du chemin brille un peu.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -8348,8 +8348,8 @@
           <t>narrateur|L'herbe garde encore la chaleur des genoux.
 enfant-m|Tu t'es assis, d'abord.
 copain|Puis le jaune est venu, tout droit.
-papa|L'élan s'est assis, puis il a guetté.
-maman|Le pré redevient calme.
+papa|Vous avez attendu, assis.
+maman|Une tige vous a chatouillés, sans rien dire.
 narrateur|Le chapeau bleu reste sur les cheveux.
 narrateur|Une graine reste coincée au tissu.
 enfant-m|À demain, les tiges.
@@ -8380,12 +8380,12 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu restes avec nous ? Un, deux, trois, on ne bouge plus. Aniss s'arrête seulement quand elle dit trois. Victorino touche le chapeau à chaque chiffre. Je peux attendre le trois ! Moi aussi, j'attends. L'herbe redevient droite, autour. Vous avez demandé, et ça marche. Mes chiffres ont tenu l'élan.</t>
+          <t>Maman, tu restes avec nous ? Chut, on écoute l'herbe. Aniss ouvre la bouche, puis la referme. Victorino tient le chapeau, sans le secouer. Je peux être silencieux ! Moi aussi, j'écoute. Un criquet reprend, tout près. Vous avez demandé, et ça tient. Mon chut a tenu vos pieds.</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu restes avec nous ? Un, deux, trois, on ne bouge plus. Aniss s'arrête seulement quand elle dit trois. Victorino touche le chapeau à chaque chiffre. Je peux attendre le trois ! Moi aussi, j'attends. L'herbe redevient droite, autour. Vous avez demandé, et ça marche. Mes chiffres ont tenu l'élan.</t>
+          <t>Maman, tu restes avec nous ? Chut, on écoute l'herbe. Aniss ouvre la bouche, puis la referme. Victorino tient le chapeau, sans le secouer. Je peux être silencieux ! Moi aussi, j'écoute. Un criquet reprend, tout près. Vous avez demandé, et ça tient. Mon chut a tenu vos pieds.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -8521,14 +8521,14 @@
       <c r="AW42" t="inlineStr">
         <is>
           <t>enfant-m|Maman, tu restes avec nous ?
-maman|Un, deux, trois, on ne bouge plus.
-narrateur|Aniss s'arrête seulement quand elle dit trois.
-narrateur|Victorino touche le chapeau à chaque chiffre.
-copain|Je peux attendre le trois !
-enfant-m|Moi aussi, j'attends.
-narrateur|L'herbe redevient droite, autour.
-papa|Vous avez demandé, et ça marche.
-maman|Mes chiffres ont tenu l'élan.</t>
+maman|Chut, on écoute l'herbe.
+narrateur|Aniss ouvre la bouche, puis la referme.
+narrateur|Victorino tient le chapeau, sans le secouer.
+copain|Je peux être silencieux !
+enfant-m|Moi aussi, j'écoute.
+narrateur|Un criquet reprend, tout près.
+papa|Vous avez demandé, et ça tient.
+maman|Mon chut a tenu vos pieds.</t>
         </is>
       </c>
     </row>
@@ -8555,12 +8555,12 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Le trois de maman reste dans l'air, tout léger. J'ai attendu le chiffre. On a demandé, et ça allait. Mes mots ont tenu vos pieds. Le pré vous rend le silence. Le chapeau bleu pose un grain de jaune sur le bois. Victorino touche la tige, du bout. Il s'est posé. Une ombre de peuplier barre encore l'herbe.</t>
+          <t>Le chut de maman reste dans l'air, tout léger. J'ai fermé la bouche. On a demandé, et ça tenait. Mon silence a tenu vos pieds. Le criquet a repris, pour vous. Le chapeau bleu pose un grain de jaune sur le bois. Victorino touche la tige, du bout. Il s'est posé. Une ombre de peuplier barre encore l'herbe.</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Le trois de maman reste dans l'air, tout léger. J'ai attendu le chiffre. On a demandé, et ça allait. Mes mots ont tenu vos pieds. Le pré vous rend le silence. Le chapeau bleu pose un grain de jaune sur le bois. Victorino touche la tige, du bout. Il s'est posé. Une ombre de peuplier barre encore l'herbe.</t>
+          <t>Le chut de maman reste dans l'air, tout léger. J'ai fermé la bouche. On a demandé, et ça tenait. Mon silence a tenu vos pieds. Le criquet a repris, pour vous. Le chapeau bleu pose un grain de jaune sur le bois. Victorino touche la tige, du bout. Il s'est posé. Une ombre de peuplier barre encore l'herbe.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -8695,11 +8695,11 @@
       <c r="AV43" s="2" t="inlineStr"/>
       <c r="AW43" t="inlineStr">
         <is>
-          <t>narrateur|Le trois de maman reste dans l'air, tout léger.
-copain|J'ai attendu le chiffre.
-enfant-m|On a demandé, et ça allait.
-maman|Mes mots ont tenu vos pieds.
-papa|Le pré vous rend le silence.
+          <t>narrateur|Le chut de maman reste dans l'air, tout léger.
+copain|J'ai fermé la bouche.
+enfant-m|On a demandé, et ça tenait.
+maman|Mon silence a tenu vos pieds.
+papa|Le criquet a repris, pour vous.
 narrateur|Le chapeau bleu pose un grain de jaune sur le bois.
 narrateur|Victorino touche la tige, du bout.
 copain|Il s'est posé.
@@ -8730,12 +8730,12 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Victorino avance, le chapeau tout bas. Les lavandes sentent partout, Aniss. Je vais jusqu'au bout, trop vite ! Ses pieds tapent les tiges, puis reviennent. Des brins collent à l'aile du chapeau. Un parfum lève, puis retombe. Il a de l'élan, comme un petit vent. Toi tu vas plus loin, lui plus vite. On peut guetter avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Victorino avance, le chapeau tout bas. Ça sent le savon et le miel, Aniss. Je pousse les tiges, trop fort ! Un nuage de parfum saute, puis retombe. Des brins collent à l'aile du chapeau. Le jaune quitte le violet, d'un coup. Tes pieds ont réveillé les fleurs. On s'approche sans les bousculer. Il peut revenir ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Victorino avance, le chapeau tout bas. Les lavandes sentent partout, Aniss. Je vais jusqu'au bout, trop vite ! Ses pieds tapent les tiges, puis reviennent. Des brins collent à l'aile du chapeau. Un parfum lève, puis retombe. Il a de l'élan, comme un petit vent. Toi tu vas plus loin, lui plus vite. On peut guetter avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Victorino avance, le chapeau tout bas. Ça sent le savon et le miel, Aniss. Je pousse les tiges, trop fort ! Un nuage de parfum saute, puis retombe. Des brins collent à l'aile du chapeau. Le jaune quitte le violet, d'un coup. Tes pieds ont réveillé les fleurs. On s'approche sans les bousculer. Il peut revenir ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -8871,14 +8871,14 @@
       <c r="AW44" t="inlineStr">
         <is>
           <t>narrateur|Victorino avance, le chapeau tout bas.
-enfant-m|Les lavandes sentent partout, Aniss.
-copain|Je vais jusqu'au bout, trop vite !
-narrateur|Ses pieds tapent les tiges, puis reviennent.
+enfant-m|Ça sent le savon et le miel, Aniss.
+copain|Je pousse les tiges, trop fort !
+narrateur|Un nuage de parfum saute, puis retombe.
 narrateur|Des brins collent à l'aile du chapeau.
-narrateur|Un parfum lève, puis retombe.
-maman|Il a de l'élan, comme un petit vent.
-papa|Toi tu vas plus loin, lui plus vite.
-enfant-m|On peut guetter avec lui ?
+narrateur|Le jaune quitte le violet, d'un coup.
+maman|Tes pieds ont réveillé les fleurs.
+papa|On s'approche sans les bousculer.
+enfant-m|Il peut revenir ?
 papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
@@ -8911,12 +8911,12 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Les lavandes bougent encore, un peu. Souffler, attendre, ou la fleur de papa ?</t>
+          <t>Le parfum tient encore, tout bas. Souffler, attendre, ou la fleur de papa ?</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Les lavandes bougent encore, un peu. Souffler, attendre, ou la fleur de papa ?</t>
+          <t>Le parfum tient encore, tout bas. Souffler, attendre, ou la fleur de papa ?</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -9075,7 +9075,7 @@
       <c r="AV45" s="2" t="inlineStr"/>
       <c r="AW45" t="inlineStr">
         <is>
-          <t>narrateur|Les lavandes bougent encore, un peu.
+          <t>narrateur|Le parfum tient encore, tout bas.
 maman|Souffler, attendre, ou la fleur de papa ?</t>
         </is>
       </c>
@@ -9103,12 +9103,12 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>On souffle tout doux. Toi derrière, moi devant ! Victorino garde le chapeau, Aniss souffle devant. Deux souffles passent sur la même tige. Aniss va plus vite, Victorino plus loin. On arrive au violet, tous les deux. J'ai attendu ton souffle, un peu. Vous avez joué avec l'élan. Les lavandes vous ont laissés passer.</t>
+          <t>On souffle tout doux. Comme le petit vent ! Victorino garde le chapeau, Aniss souffle devant. Deux souffles passent sur la même tige. Le violet penche, puis se redresse. On n'a rien cassé. J'ai soufflé plus bas, cette fois. Vous avez joué avec l'air. Les fleurs sont restées debout.</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>On souffle tout doux. Toi derrière, moi devant ! Victorino garde le chapeau, Aniss souffle devant. Deux souffles passent sur la même tige. Aniss va plus vite, Victorino plus loin. On arrive au violet, tous les deux. J'ai attendu ton souffle, un peu. Vous avez joué avec l'élan. Les lavandes vous ont laissés passer.</t>
+          <t>On souffle tout doux. Comme le petit vent ! Victorino garde le chapeau, Aniss souffle devant. Deux souffles passent sur la même tige. Le violet penche, puis se redresse. On n'a rien cassé. J'ai soufflé plus bas, cette fois. Vous avez joué avec l'air. Les fleurs sont restées debout.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -9244,14 +9244,14 @@
       <c r="AW46" t="inlineStr">
         <is>
           <t>enfant-m|On souffle tout doux.
-copain|Toi derrière, moi devant !
+copain|Comme le petit vent !
 narrateur|Victorino garde le chapeau, Aniss souffle devant.
 narrateur|Deux souffles passent sur la même tige.
-narrateur|Aniss va plus vite, Victorino plus loin.
-enfant-m|On arrive au violet, tous les deux.
-copain|J'ai attendu ton souffle, un peu.
-papa|Vous avez joué avec l'élan.
-maman|Les lavandes vous ont laissés passer.</t>
+narrateur|Le violet penche, puis se redresse.
+enfant-m|On n'a rien cassé.
+copain|J'ai soufflé plus bas, cette fois.
+papa|Vous avez joué avec l'air.
+maman|Les fleurs sont restées debout.</t>
         </is>
       </c>
     </row>
@@ -9278,12 +9278,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Deux souffles marquent la même tige violette. Toi devant, moi derrière. Tes pas allaient plus loin. Vous avez soufflé avec l'élan, pas contre. Les lavandes redeviennent tièdes, et calmes. Le chapeau bleu reste sur les cheveux. Un brin violet sèche déjà sur le tissu. On rentre, le parfum reste. Le puits fait une ombre ronde.</t>
+          <t>Deux souffles marquent la même tige violette. On n'a rien cassé. J'ai soufflé plus bas. Vous avez joué avec l'air. Les lavandes sont encore debout. Le chapeau bleu reste sur les cheveux. Un brin violet sèche déjà sur le tissu. Le parfum rentre avec nous. Le puits fait une ombre ronde.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Deux souffles marquent la même tige violette. Toi devant, moi derrière. Tes pas allaient plus loin. Vous avez soufflé avec l'élan, pas contre. Les lavandes redeviennent tièdes, et calmes. Le chapeau bleu reste sur les cheveux. Un brin violet sèche déjà sur le tissu. On rentre, le parfum reste. Le puits fait une ombre ronde.</t>
+          <t>Deux souffles marquent la même tige violette. On n'a rien cassé. J'ai soufflé plus bas. Vous avez joué avec l'air. Les lavandes sont encore debout. Le chapeau bleu reste sur les cheveux. Un brin violet sèche déjà sur le tissu. Le parfum rentre avec nous. Le puits fait une ombre ronde.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -9419,13 +9419,13 @@
       <c r="AW47" t="inlineStr">
         <is>
           <t>narrateur|Deux souffles marquent la même tige violette.
-enfant-m|Toi devant, moi derrière.
-copain|Tes pas allaient plus loin.
-papa|Vous avez soufflé avec l'élan, pas contre.
-maman|Les lavandes redeviennent tièdes, et calmes.
+enfant-m|On n'a rien cassé.
+copain|J'ai soufflé plus bas.
+papa|Vous avez joué avec l'air.
+maman|Les lavandes sont encore debout.
 narrateur|Le chapeau bleu reste sur les cheveux.
 narrateur|Un brin violet sèche déjà sur le tissu.
-enfant-m|On rentre, le parfum reste.
+enfant-m|Le parfum rentre avec nous.
 narrateur|Le puits fait une ombre ronde.</t>
         </is>
       </c>
@@ -9453,12 +9453,12 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>J'attends le parfum. Moi je finis, puis c'est toi. Victorino tient le chapeau, sans le bouger. Aniss tapote une tige, tout seul d'abord. Il souffle, puis il recule. C'est à toi, Victorino. Merci, j'y vais. Chacun son tour, entre les tiges. L'élan a attendu le parfum.</t>
+          <t>J'attends le parfum. Quand il retombe, on avance. Victorino tient le chapeau, sans le bouger. Aniss compte les tiges, tout bas. Le nuage violet s'assoit, enfin. C'est à toi, Victorino. Merci, j'y vais. Le parfum vous a fait de la place. Vous l'avez laissé se poser.</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>J'attends le parfum. Moi je finis, puis c'est toi. Victorino tient le chapeau, sans le bouger. Aniss tapote une tige, tout seul d'abord. Il souffle, puis il recule. C'est à toi, Victorino. Merci, j'y vais. Chacun son tour, entre les tiges. L'élan a attendu le parfum.</t>
+          <t>J'attends le parfum. Quand il retombe, on avance. Victorino tient le chapeau, sans le bouger. Aniss compte les tiges, tout bas. Le nuage violet s'assoit, enfin. C'est à toi, Victorino. Merci, j'y vais. Le parfum vous a fait de la place. Vous l'avez laissé se poser.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -9594,14 +9594,14 @@
       <c r="AW48" t="inlineStr">
         <is>
           <t>enfant-m|J'attends le parfum.
-copain|Moi je finis, puis c'est toi.
+copain|Quand il retombe, on avance.
 narrateur|Victorino tient le chapeau, sans le bouger.
-narrateur|Aniss tapote une tige, tout seul d'abord.
-narrateur|Il souffle, puis il recule.
+narrateur|Aniss compte les tiges, tout bas.
+narrateur|Le nuage violet s'assoit, enfin.
 copain|C'est à toi, Victorino.
 enfant-m|Merci, j'y vais.
-papa|Chacun son tour, entre les tiges.
-maman|L'élan a attendu le parfum.</t>
+papa|Le parfum vous a fait de la place.
+maman|Vous l'avez laissé se poser.</t>
         </is>
       </c>
     </row>
@@ -9628,12 +9628,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Le parfum attend encore, tout bas. J'ai fini, puis c'était toi. J'ai attendu ta tige. Chacun son tour, entre les tiges. L'élan a laissé la place. Le chapeau bleu garde un grain de parfum. Victorino souffle dessus, tout doux. On se dit au revoir, lavandes. Une abeille passe, sans se presser.</t>
+          <t>Le parfum s'est assis, tout bas. Quand il est retombé, on a avancé. J'ai attendu ta tige. Le nuage vous a laissés passer. Vous l'avez laissé se poser. Le chapeau bleu garde un grain de parfum. Victorino souffle dessus, tout doux. Au revoir, les tiges. Une abeille passe, sans se presser.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Le parfum attend encore, tout bas. J'ai fini, puis c'était toi. J'ai attendu ta tige. Chacun son tour, entre les tiges. L'élan a laissé la place. Le chapeau bleu garde un grain de parfum. Victorino souffle dessus, tout doux. On se dit au revoir, lavandes. Une abeille passe, sans se presser.</t>
+          <t>Le parfum s'est assis, tout bas. Quand il est retombé, on a avancé. J'ai attendu ta tige. Le nuage vous a laissés passer. Vous l'avez laissé se poser. Le chapeau bleu garde un grain de parfum. Victorino souffle dessus, tout doux. Au revoir, les tiges. Une abeille passe, sans se presser.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -9768,14 +9768,14 @@
       <c r="AV49" s="2" t="inlineStr"/>
       <c r="AW49" t="inlineStr">
         <is>
-          <t>narrateur|Le parfum attend encore, tout bas.
-copain|J'ai fini, puis c'était toi.
+          <t>narrateur|Le parfum s'est assis, tout bas.
+copain|Quand il est retombé, on a avancé.
 enfant-m|J'ai attendu ta tige.
-maman|Chacun son tour, entre les tiges.
-papa|L'élan a laissé la place.
+maman|Le nuage vous a laissés passer.
+papa|Vous l'avez laissé se poser.
 narrateur|Le chapeau bleu garde un grain de parfum.
 narrateur|Victorino souffle dessus, tout doux.
-copain|On se dit au revoir, lavandes.
+copain|Au revoir, les tiges.
 narrateur|Une abeille passe, sans se presser.</t>
         </is>
       </c>
@@ -9803,12 +9803,12 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu gardes la fleur ? Je la tends, un pas chacun. Papa pose la fleur près du chapeau. Aniss s'approche, tout petit pas. Victorino s'approche, encore plus lent. On demande, et ça va ! Le violet est à nous. Vous avez demandé, tout calme. Ma main a juste attendu.</t>
+          <t>Papa, tu gardes la fleur ? Je la tends, un pas chacun. Papa pose la fleur près du chapeau. Aniss pose un pied, puis l'autre. Victorino pose le même pas, plus tard. On a demandé, et ça va ! Le violet est tout près. Vous avez demandé, tout calme. Ma main n'a pas bougé.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu gardes la fleur ? Je la tends, un pas chacun. Papa pose la fleur près du chapeau. Aniss s'approche, tout petit pas. Victorino s'approche, encore plus lent. On demande, et ça va ! Le violet est à nous. Vous avez demandé, tout calme. Ma main a juste attendu.</t>
+          <t>Papa, tu gardes la fleur ? Je la tends, un pas chacun. Papa pose la fleur près du chapeau. Aniss pose un pied, puis l'autre. Victorino pose le même pas, plus tard. On a demandé, et ça va ! Le violet est tout près. Vous avez demandé, tout calme. Ma main n'a pas bougé.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -9946,12 +9946,12 @@
           <t>enfant-m|Papa, tu gardes la fleur ?
 papa|Je la tends, un pas chacun.
 narrateur|Papa pose la fleur près du chapeau.
-narrateur|Aniss s'approche, tout petit pas.
-narrateur|Victorino s'approche, encore plus lent.
-copain|On demande, et ça va !
-enfant-m|Le violet est à nous.
+narrateur|Aniss pose un pied, puis l'autre.
+narrateur|Victorino pose le même pas, plus tard.
+copain|On a demandé, et ça va !
+enfant-m|Le violet est tout près.
 maman|Vous avez demandé, tout calme.
-papa|Ma main a juste attendu.</t>
+papa|Ma main n'a pas bougé.</t>
         </is>
       </c>
     </row>
@@ -9978,12 +9978,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>La fleur de papa repose près du violet. Tu la tendais, un pas chacun. On a demandé, et ça venait juste. Ma main a fait le tour, rien de plus. Les lavandes ont rendu le jaune. Le chapeau bleu reste sur les cheveux. Un rond clair reste sur une feuille. Regarde, Aniss, il brille. Le chat reprend la pierre, au frais.</t>
+          <t>La fleur de papa repose près du violet. Tu la tendais, un pas chacun. On a demandé, et ça venait juste. Ma main n'a pas bougé. Les lavandes ont rendu le jaune. Le chapeau bleu reste sur les cheveux. Un rond clair reste sur une feuille. Regarde, Aniss, il brille. Le chat reprend la pierre, au frais.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>La fleur de papa repose près du violet. Tu la tendais, un pas chacun. On a demandé, et ça venait juste. Ma main a fait le tour, rien de plus. Les lavandes ont rendu le jaune. Le chapeau bleu reste sur les cheveux. Un rond clair reste sur une feuille. Regarde, Aniss, il brille. Le chat reprend la pierre, au frais.</t>
+          <t>La fleur de papa repose près du violet. Tu la tendais, un pas chacun. On a demandé, et ça venait juste. Ma main n'a pas bougé. Les lavandes ont rendu le jaune. Le chapeau bleu reste sur les cheveux. Un rond clair reste sur une feuille. Regarde, Aniss, il brille. Le chat reprend la pierre, au frais.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -10121,7 +10121,7 @@
           <t>narrateur|La fleur de papa repose près du violet.
 enfant-m|Tu la tendais, un pas chacun.
 copain|On a demandé, et ça venait juste.
-papa|Ma main a fait le tour, rien de plus.
+papa|Ma main n'a pas bougé.
 maman|Les lavandes ont rendu le jaune.
 narrateur|Le chapeau bleu reste sur les cheveux.
 narrateur|Un rond clair reste sur une feuille.
@@ -10153,12 +10153,12 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Le chapeau bleu frôle le muret chaud. Ici, la pierre est chaude, Aniss. J'entends mes pieds deux fois ! Le muret renvoie chaque pas, tout fort. Le bord du chapeau tape la pierre. Le chapeau bleu attend au bord, un peu seule. Son élan remplit toute la pierre. Toi tu vas plus loin, lui plus vite. On guette comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Le chapeau bleu frôle le muret chaud. La pierre est tiède, Aniss. J'entends mes pieds deux fois ! Chaque clic revient, plus fort. Le bord du chapeau tape la pierre. Le chapeau bleu n'ose plus bouger. Le jaune n'aime pas le bruit. La pierre répète tes pas. On fait moins de clic ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>Le chapeau bleu frôle le muret chaud. Ici, la pierre est chaude, Aniss. J'entends mes pieds deux fois ! Le muret renvoie chaque pas, tout fort. Le bord du chapeau tape la pierre. Le chapeau bleu attend au bord, un peu seule. Son élan remplit toute la pierre. Toi tu vas plus loin, lui plus vite. On guette comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>Le chapeau bleu frôle le muret chaud. La pierre est tiède, Aniss. J'entends mes pieds deux fois ! Chaque clic revient, plus fort. Le bord du chapeau tape la pierre. Le chapeau bleu n'ose plus bouger. Le jaune n'aime pas le bruit. La pierre répète tes pas. On fait moins de clic ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -10294,14 +10294,14 @@
       <c r="AW52" t="inlineStr">
         <is>
           <t>narrateur|Le chapeau bleu frôle le muret chaud.
-enfant-m|Ici, la pierre est chaude, Aniss.
+enfant-m|La pierre est tiède, Aniss.
 copain|J'entends mes pieds deux fois !
-narrateur|Le muret renvoie chaque pas, tout fort.
+narrateur|Chaque clic revient, plus fort.
 narrateur|Le bord du chapeau tape la pierre.
-narrateur|Le chapeau bleu attend au bord, un peu seule.
-maman|Son élan remplit toute la pierre.
-papa|Toi tu vas plus loin, lui plus vite.
-copain|On guette comment, alors ?
+narrateur|Le chapeau bleu n'ose plus bouger.
+maman|Le jaune n'aime pas le bruit.
+papa|La pierre répète tes pas.
+copain|On fait moins de clic ?
 papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
@@ -10329,12 +10329,12 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Les clics remplissent encore le muret. Le rythme, en bas, ou la main de maman ?</t>
+          <t>Un dernier clic roule le long du muret. Le rythme, en bas, ou la main de maman ?</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>Les clics remplissent encore le muret. Le rythme, en bas, ou la main de maman ?</t>
+          <t>Un dernier clic roule le long du muret. Le rythme, en bas, ou la main de maman ?</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -10493,7 +10493,7 @@
       <c r="AV53" s="2" t="inlineStr"/>
       <c r="AW53" t="inlineStr">
         <is>
-          <t>narrateur|Les clics remplissent encore le muret.
+          <t>narrateur|Un dernier clic roule le long du muret.
 papa|Le rythme, en bas, ou la main de maman ?</t>
         </is>
       </c>
@@ -10521,12 +10521,12 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>On fait un rythme sur la pierre. Toc toc, j'avance ! Victorino pose une main sur l'épaule d'Aniss. Le chapeau bleu voyage sur les cheveux, entre deux taps. Ils tapent la même pierre, l'un après l'autre. Doucement, le rythme tient. Le clic suit le rythme, puis se tait. Vous jouez avec le bruit, ensemble. Le muret est devenu un tambour.</t>
+          <t>On tape une fois, puis plus. Toc, et j'attends. Victorino pose une main sur l'épaule d'Aniss. Le chapeau bleu s'arrête après le dernier toc. La pierre répond, puis se tait. Le jaune aime le silence, après. Moi aussi, après le toc. Vous avez joué avec le bruit. Un toc, puis la pierre dort.</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>On fait un rythme sur la pierre. Toc toc, j'avance ! Victorino pose une main sur l'épaule d'Aniss. Le chapeau bleu voyage sur les cheveux, entre deux taps. Ils tapent la même pierre, l'un après l'autre. Doucement, le rythme tient. Le clic suit le rythme, puis se tait. Vous jouez avec le bruit, ensemble. Le muret est devenu un tambour.</t>
+          <t>On tape une fois, puis plus. Toc, et j'attends. Victorino pose une main sur l'épaule d'Aniss. Le chapeau bleu s'arrête après le dernier toc. La pierre répond, puis se tait. Le jaune aime le silence, après. Moi aussi, après le toc. Vous avez joué avec le bruit. Un toc, puis la pierre dort.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -10661,15 +10661,15 @@
       <c r="AV54" s="2" t="inlineStr"/>
       <c r="AW54" t="inlineStr">
         <is>
-          <t>enfant-m|On fait un rythme sur la pierre.
-copain|Toc toc, j'avance !
+          <t>enfant-m|On tape une fois, puis plus.
+copain|Toc, et j'attends.
 narrateur|Victorino pose une main sur l'épaule d'Aniss.
-narrateur|Le chapeau bleu voyage sur les cheveux, entre deux taps.
-narrateur|Ils tapent la même pierre, l'un après l'autre.
-enfant-m|Doucement, le rythme tient.
-copain|Le clic suit le rythme, puis se tait.
-papa|Vous jouez avec le bruit, ensemble.
-maman|Le muret est devenu un tambour.</t>
+narrateur|Le chapeau bleu s'arrête après le dernier toc.
+narrateur|La pierre répond, puis se tait.
+enfant-m|Le jaune aime le silence, après.
+copain|Moi aussi, après le toc.
+papa|Vous avez joué avec le bruit.
+maman|Un toc, puis la pierre dort.</t>
         </is>
       </c>
     </row>
@@ -10696,12 +10696,12 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Le rythme s'arrête, et le jaune se pose. Toc toc, on est arrivés. J'avais la main sur ton épaule. Le muret est redevenu une pierre, simplement. Le clic s'est couché. Le chapeau bleu reste sur les cheveux. Une poussière tourne encore, puis tombe. On rentre, le tambour se tait. Dehors, le pré redevient calme.</t>
+          <t>Après le toc, le jaune se pose. J'ai tapé une fois, puis plus. J'avais la main sur ton épaule. La pierre a fini par dormir. Un toc, puis le silence. Le chapeau bleu reste sur les cheveux. Une poussière tourne encore, puis tombe. Le muret s'est tu. Dehors, le pré redevient calme.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Le rythme s'arrête, et le jaune se pose. Toc toc, on est arrivés. J'avais la main sur ton épaule. Le muret est redevenu une pierre, simplement. Le clic s'est couché. Le chapeau bleu reste sur les cheveux. Une poussière tourne encore, puis tombe. On rentre, le tambour se tait. Dehors, le pré redevient calme.</t>
+          <t>Après le toc, le jaune se pose. J'ai tapé une fois, puis plus. J'avais la main sur ton épaule. La pierre a fini par dormir. Un toc, puis le silence. Le chapeau bleu reste sur les cheveux. Une poussière tourne encore, puis tombe. Le muret s'est tu. Dehors, le pré redevient calme.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -10836,14 +10836,14 @@
       <c r="AV55" s="2" t="inlineStr"/>
       <c r="AW55" t="inlineStr">
         <is>
-          <t>narrateur|Le rythme s'arrête, et le jaune se pose.
-copain|Toc toc, on est arrivés.
+          <t>narrateur|Après le toc, le jaune se pose.
+copain|J'ai tapé une fois, puis plus.
 enfant-m|J'avais la main sur ton épaule.
-papa|Le muret est redevenu une pierre, simplement.
-maman|Le clic s'est couché.
+papa|La pierre a fini par dormir.
+maman|Un toc, puis le silence.
 narrateur|Le chapeau bleu reste sur les cheveux.
 narrateur|Une poussière tourne encore, puis tombe.
-enfant-m|On rentre, le tambour se tait.
+enfant-m|Le muret s'est tu.
 narrateur|Dehors, le pré redevient calme.</t>
         </is>
       </c>
@@ -10871,12 +10871,12 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>On attend en bas. Quand la pierre se tait, je m'approche. Un pas dans l'herbe, puis plus rien. Le chapeau bleu reste muet, au creux. Le muret se tait, enfin. Maintenant ! À toi, puis à moi. Vous avez laissé le bruit s'asseoir. L'élan a attendu le silence.</t>
+          <t>On attend en bas. La pierre se tait, d'abord. Leurs chaussures restent dans l'herbe fraîche. Le chapeau bleu reste dans l'ombre, en bas. Le muret ne clique plus. Maintenant, on peut regarder. À toi, puis à moi. Vous avez laissé le bruit s'en aller. En bas, vos pieds sont plus doux.</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>On attend en bas. Quand la pierre se tait, je m'approche. Un pas dans l'herbe, puis plus rien. Le chapeau bleu reste muet, au creux. Le muret se tait, enfin. Maintenant ! À toi, puis à moi. Vous avez laissé le bruit s'asseoir. L'élan a attendu le silence.</t>
+          <t>On attend en bas. La pierre se tait, d'abord. Leurs chaussures restent dans l'herbe fraîche. Le chapeau bleu reste dans l'ombre, en bas. Le muret ne clique plus. Maintenant, on peut regarder. À toi, puis à moi. Vous avez laissé le bruit s'en aller. En bas, vos pieds sont plus doux.</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -11012,14 +11012,14 @@
       <c r="AW56" t="inlineStr">
         <is>
           <t>enfant-m|On attend en bas.
-copain|Quand la pierre se tait, je m'approche.
-narrateur|Un pas dans l'herbe, puis plus rien.
-narrateur|Le chapeau bleu reste muet, au creux.
-narrateur|Le muret se tait, enfin.
-copain|Maintenant !
+copain|La pierre se tait, d'abord.
+narrateur|Leurs chaussures restent dans l'herbe fraîche.
+narrateur|Le chapeau bleu reste dans l'ombre, en bas.
+narrateur|Le muret ne clique plus.
+copain|Maintenant, on peut regarder.
 enfant-m|À toi, puis à moi.
-papa|Vous avez laissé le bruit s'asseoir.
-maman|L'élan a attendu le silence.</t>
+papa|Vous avez laissé le bruit s'en aller.
+maman|En bas, vos pieds sont plus doux.</t>
         </is>
       </c>
     </row>
@@ -11046,12 +11046,12 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>La pierre s'est tue, enfin, tout à fait. On a attendu en bas. Quand elle était partie, on s'approchait. Le silence vous a laissé le jaune. L'élan a écouté la pierre. Le chapeau bleu ne fait plus aucun bruit. Victorino pose la paume sur la pierre chaude. Elle est tiède. Un oiseau passe au-dessus du muret, sans crier.</t>
+          <t>La pierre s'est tue, enfin, tout à fait. On a attendu en bas. Nos chaussures sont restées dans l'herbe. Le silence vous a laissé le jaune. En bas, vos pieds étaient plus doux. Le chapeau bleu ne fait plus aucun bruit. Victorino pose la paume sur la pierre chaude. Elle est tiède. Un oiseau passe au-dessus du muret, sans crier.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>La pierre s'est tue, enfin, tout à fait. On a attendu en bas. Quand elle était partie, on s'approchait. Le silence vous a laissé le jaune. L'élan a écouté la pierre. Le chapeau bleu ne fait plus aucun bruit. Victorino pose la paume sur la pierre chaude. Elle est tiède. Un oiseau passe au-dessus du muret, sans crier.</t>
+          <t>La pierre s'est tue, enfin, tout à fait. On a attendu en bas. Nos chaussures sont restées dans l'herbe. Le silence vous a laissé le jaune. En bas, vos pieds étaient plus doux. Le chapeau bleu ne fait plus aucun bruit. Victorino pose la paume sur la pierre chaude. Elle est tiède. Un oiseau passe au-dessus du muret, sans crier.</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -11188,9 +11188,9 @@
         <is>
           <t>narrateur|La pierre s'est tue, enfin, tout à fait.
 enfant-m|On a attendu en bas.
-copain|Quand elle était partie, on s'approchait.
+copain|Nos chaussures sont restées dans l'herbe.
 papa|Le silence vous a laissé le jaune.
-maman|L'élan a écouté la pierre.
+maman|En bas, vos pieds étaient plus doux.
 narrateur|Le chapeau bleu ne fait plus aucun bruit.
 narrateur|Victorino pose la paume sur la pierre chaude.
 copain|Elle est tiède.
@@ -11221,12 +11221,12 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tends la main ? Je reste, et vous venez tout doux. Aniss écoute la paume, plus que ses pieds. Victorino touche le chapeau quand maman ouvre la paume. Je m'arrête sur ta main ! Moi aussi, j'écoute. Le clic se range derrière le silence. Vous avez demandé la main. Ma paume a tenu l'élan.</t>
+          <t>Maman, tu tends la main ? Je reste, et vous venez tout doux. Aniss regarde la paume, plus que ses pieds. Victorino touche le chapeau quand maman ouvre la paume. Je m'arrête devant ta main ! Moi aussi, j'écoute. Un grain de foin dort dans ses plis. Vous avez demandé la main. Ma paume est devenue une tige.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tends la main ? Je reste, et vous venez tout doux. Aniss écoute la paume, plus que ses pieds. Victorino touche le chapeau quand maman ouvre la paume. Je m'arrête sur ta main ! Moi aussi, j'écoute. Le clic se range derrière le silence. Vous avez demandé la main. Ma paume a tenu l'élan.</t>
+          <t>Maman, tu tends la main ? Je reste, et vous venez tout doux. Aniss regarde la paume, plus que ses pieds. Victorino touche le chapeau quand maman ouvre la paume. Je m'arrête devant ta main ! Moi aussi, j'écoute. Un grain de foin dort dans ses plis. Vous avez demandé la main. Ma paume est devenue une tige.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -11363,13 +11363,13 @@
         <is>
           <t>enfant-m|Maman, tu tends la main ?
 maman|Je reste, et vous venez tout doux.
-narrateur|Aniss écoute la paume, plus que ses pieds.
+narrateur|Aniss regarde la paume, plus que ses pieds.
 narrateur|Victorino touche le chapeau quand maman ouvre la paume.
-copain|Je m'arrête sur ta main !
+copain|Je m'arrête devant ta main !
 enfant-m|Moi aussi, j'écoute.
-narrateur|Le clic se range derrière le silence.
+narrateur|Un grain de foin dort dans ses plis.
 papa|Vous avez demandé la main.
-maman|Ma paume a tenu l'élan.</t>
+maman|Ma paume est devenue une tige.</t>
         </is>
       </c>
     </row>
@@ -11396,12 +11396,12 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>La paume de maman s'ouvre, puis se referme. J'écoutais ta main. Moi aussi, je m'arrêtais dessus. Vous avez demandé le calme. Le muret a rendu vos pas. Le chapeau bleu reste sur les cheveux. Victorino touche la pierre, du bout des doigts. Il s'est posé, Aniss. La pierre garde une poussière, puis plus rien.</t>
+          <t>La paume de maman s'ouvre, puis se referme. J'écoutais ta main. Moi aussi, je m'arrêtais dessus. Vous avez demandé le calme. Un grain de foin reste dans ses plis. Le chapeau bleu reste sur les cheveux. Victorino touche la pierre, du bout des doigts. Il s'est posé, Aniss. La pierre garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>La paume de maman s'ouvre, puis se referme. J'écoutais ta main. Moi aussi, je m'arrêtais dessus. Vous avez demandé le calme. Le muret a rendu vos pas. Le chapeau bleu reste sur les cheveux. Victorino touche la pierre, du bout des doigts. Il s'est posé, Aniss. La pierre garde une poussière, puis plus rien.</t>
+          <t>La paume de maman s'ouvre, puis se referme. J'écoutais ta main. Moi aussi, je m'arrêtais dessus. Vous avez demandé le calme. Un grain de foin reste dans ses plis. Le chapeau bleu reste sur les cheveux. Victorino touche la pierre, du bout des doigts. Il s'est posé, Aniss. La pierre garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -11540,7 +11540,7 @@
 enfant-m|J'écoutais ta main.
 copain|Moi aussi, je m'arrêtais dessus.
 maman|Vous avez demandé le calme.
-papa|Le muret a rendu vos pas.
+papa|Un grain de foin reste dans ses plis.
 narrateur|Le chapeau bleu reste sur les cheveux.
 narrateur|Victorino touche la pierre, du bout des doigts.
 enfant-m|Il s'est posé, Aniss.
@@ -11933,12 +11933,12 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>La poche cache encore le papier plié. Ça sent la colle. La fleur attend le jaune. Le manteau d'Aniss s'arrête trop haut. Les manches laissent ses poignets libres. Le pré est tiède, devant. On y va, tous les quatre ? Oui.</t>
+          <t>La poche garde le papier, tout plat. Ça sent encore la colle. Le jaune va croire que c'est vrai. Les poignets d'Aniss dépassent des manches. Il frappe deux fois le portail, pour rien. Le pré vous attend, tout tiède. On ouvre, tous les quatre ? Oui.</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>La poche cache encore le papier plié. Ça sent la colle. La fleur attend le jaune. Le manteau d'Aniss s'arrête trop haut. Les manches laissent ses poignets libres. Le pré est tiède, devant. On y va, tous les quatre ? Oui.</t>
+          <t>La poche garde le papier, tout plat. Ça sent encore la colle. Le jaune va croire que c'est vrai. Les poignets d'Aniss dépassent des manches. Il frappe deux fois le portail, pour rien. Le pré vous attend, tout tiède. On ouvre, tous les quatre ? Oui.</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -12077,13 +12077,13 @@
       </c>
       <c r="AW62" t="inlineStr">
         <is>
-          <t>narrateur|La poche cache encore le papier plié.
-copain|Ça sent la colle.
-enfant-m|La fleur attend le jaune.
-narrateur|Le manteau d'Aniss s'arrête trop haut.
-narrateur|Les manches laissent ses poignets libres.
-maman|Le pré est tiède, devant.
-papa|On y va, tous les quatre ?
+          <t>narrateur|La poche garde le papier, tout plat.
+copain|Ça sent encore la colle.
+enfant-m|Le jaune va croire que c'est vrai.
+narrateur|Les poignets d'Aniss dépassent des manches.
+narrateur|Il frappe deux fois le portail, pour rien.
+maman|Le pré vous attend, tout tiède.
+papa|On ouvre, tous les quatre ?
 enfant-m|Oui.</t>
         </is>
       </c>
@@ -12111,12 +12111,12 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Aniss tapote déjà le sol, tout léger. Le pré a l'herbe haute, encore tiède. Les lavandes sentent fort, tout bas. Le muret garde une pierre chaude. On commence où, pour le papillon ?</t>
+          <t>Aniss tape déjà deux cailloux, l'un contre l'autre. Le pré ondule, plus loin que le puits. Les lavandes font un mur violet, tout bas. Le muret tient encore la chaleur du chat. On guette où, d'abord ?</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>Aniss tapote déjà le sol, tout léger. Le pré a l'herbe haute, encore tiède. Les lavandes sentent fort, tout bas. Le muret garde une pierre chaude. On commence où, pour le papillon ?</t>
+          <t>Aniss tape déjà deux cailloux, l'un contre l'autre. Le pré ondule, plus loin que le puits. Les lavandes font un mur violet, tout bas. Le muret tient encore la chaleur du chat. On guette où, d'abord ?</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -12275,11 +12275,11 @@
       <c r="AV63" s="2" t="inlineStr"/>
       <c r="AW63" t="inlineStr">
         <is>
-          <t>narrateur|Aniss tapote déjà le sol, tout léger.
-narrateur|Le pré a l'herbe haute, encore tiède.
-narrateur|Les lavandes sentent fort, tout bas.
-narrateur|Le muret garde une pierre chaude.
-papa|On commence où, pour le papillon ?</t>
+          <t>narrateur|Aniss tape déjà deux cailloux, l'un contre l'autre.
+narrateur|Le pré ondule, plus loin que le puits.
+narrateur|Les lavandes font un mur violet, tout bas.
+narrateur|Le muret tient encore la chaleur du chat.
+papa|On guette où, d'abord ?</t>
         </is>
       </c>
     </row>
@@ -12306,12 +12306,12 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Victorino pose la fleur sur une tige. L'herbe du pré sent le foin chaud. Moi je cours, Victorino ! Aniss fend l'herbe, trop vite. Un nuage de graines s'envole, tout haut. La fleur se plie contre un genou. La fleur de papier n'attendait pas ça. Il a envie de bouger, c'est tout. Ses jambes sont plus courtes, plus vives. On guette comment, alors ? Vous faites comment, tous les deux ?</t>
+          <t>Victorino pose la fleur sur une tige. Les tiges se touchent, puis se séparent. Je le rattrape ! Aniss part dans l'herbe, trop loin. Le jaune s'envole, plus haut que leurs têtes. La fleur se plie contre un genou. La fleur de papier n'a pas suffi. Il a envie de courir, c'est tout. Tes pieds vont trop vite, Aniss. Je fais comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>Victorino pose la fleur sur une tige. L'herbe du pré sent le foin chaud. Moi je cours, Victorino ! Aniss fend l'herbe, trop vite. Un nuage de graines s'envole, tout haut. La fleur se plie contre un genou. La fleur de papier n'attendait pas ça. Il a envie de bouger, c'est tout. Ses jambes sont plus courtes, plus vives. On guette comment, alors ? Vous faites comment, tous les deux ?</t>
+          <t>Victorino pose la fleur sur une tige. Les tiges se touchent, puis se séparent. Je le rattrape ! Aniss part dans l'herbe, trop loin. Le jaune s'envole, plus haut que leurs têtes. La fleur se plie contre un genou. La fleur de papier n'a pas suffi. Il a envie de courir, c'est tout. Tes pieds vont trop vite, Aniss. Je fais comment, alors ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -12447,16 +12447,16 @@
       <c r="AW64" t="inlineStr">
         <is>
           <t>narrateur|Victorino pose la fleur sur une tige.
-narrateur|L'herbe du pré sent le foin chaud.
-copain|Moi je cours, Victorino !
-narrateur|Aniss fend l'herbe, trop vite.
-narrateur|Un nuage de graines s'envole, tout haut.
+narrateur|Les tiges se touchent, puis se séparent.
+copain|Je le rattrape !
+narrateur|Aniss part dans l'herbe, trop loin.
+narrateur|Le jaune s'envole, plus haut que leurs têtes.
 narrateur|La fleur se plie contre un genou.
-enfant-m|La fleur de papier n'attendait pas ça.
-maman|Il a envie de bouger, c'est tout.
-papa|Ses jambes sont plus courtes, plus vives.
-copain|On guette comment, alors ?
-papa|Vous faites comment, tous les deux ?</t>
+enfant-m|La fleur de papier n'a pas suffi.
+maman|Il a envie de courir, c'est tout.
+papa|Tes pieds vont trop vite, Aniss.
+copain|Je fais comment, alors ?
+papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="AX64" t="inlineStr">
@@ -12488,12 +12488,12 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Aniss fend encore l'herbe, tout léger. Marcher comme lui, s'asseoir, ou maman ?</t>
+          <t>L'herbe se referme derrière Aniss. Marcher comme lui, s'asseoir, ou le silence ?</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Aniss fend encore l'herbe, tout léger. Marcher comme lui, s'asseoir, ou maman ?</t>
+          <t>L'herbe se referme derrière Aniss. Marcher comme lui, s'asseoir, ou le silence ?</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -12652,8 +12652,8 @@
       <c r="AV65" s="2" t="inlineStr"/>
       <c r="AW65" t="inlineStr">
         <is>
-          <t>narrateur|Aniss fend encore l'herbe, tout léger.
-papa|Marcher comme lui, s'asseoir, ou maman ?</t>
+          <t>narrateur|L'herbe se referme derrière Aniss.
+papa|Marcher comme lui, s'asseoir, ou le silence ?</t>
         </is>
       </c>
     </row>
@@ -12680,12 +12680,12 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>On marche comme lui. Moi je bats des bras, tout lent. Aniss tient le sac, Victorino lève la fleur. Deux ombres avancent dans l'herbe, sans courir. Aniss lève un pied, puis s'arrête. Maintenant c'est moi. Puis c'est moi encore. Vous jouez à son pas. L'élan a trouvé sa place.</t>
+          <t>On marche comme lui. Moi je bats des bras, tout lent. La fleur se lève, se pose, se lève. Deux ombres avancent dans l'herbe, sans courir. Aniss lève un pied, puis le repose. Le jaune a des ailes comme ça. Les miennes aussi, maintenant. Vous jouez à son pas. Le pré vous a laissés entrer.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>On marche comme lui. Moi je bats des bras, tout lent. Aniss tient le sac, Victorino lève la fleur. Deux ombres avancent dans l'herbe, sans courir. Aniss lève un pied, puis s'arrête. Maintenant c'est moi. Puis c'est moi encore. Vous jouez à son pas. L'élan a trouvé sa place.</t>
+          <t>On marche comme lui. Moi je bats des bras, tout lent. La fleur se lève, se pose, se lève. Deux ombres avancent dans l'herbe, sans courir. Aniss lève un pied, puis le repose. Le jaune a des ailes comme ça. Les miennes aussi, maintenant. Vous jouez à son pas. Le pré vous a laissés entrer.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -12822,13 +12822,13 @@
         <is>
           <t>enfant-m|On marche comme lui.
 copain|Moi je bats des bras, tout lent.
-narrateur|Aniss tient le sac, Victorino lève la fleur.
+narrateur|La fleur se lève, se pose, se lève.
 narrateur|Deux ombres avancent dans l'herbe, sans courir.
-narrateur|Aniss lève un pied, puis s'arrête.
-enfant-m|Maintenant c'est moi.
-copain|Puis c'est moi encore.
+narrateur|Aniss lève un pied, puis le repose.
+enfant-m|Le jaune a des ailes comme ça.
+copain|Les miennes aussi, maintenant.
 papa|Vous jouez à son pas.
-maman|L'élan a trouvé sa place.</t>
+maman|Le pré vous a laissés entrer.</t>
         </is>
       </c>
     </row>
@@ -12855,12 +12855,12 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Le papillon jaune se pose, au bout d'une tige. On a marché, chacun son tour. Tu battais des bras, moi j'avançais. Vous avez laissé l'élan dessiner. Le pré sent encore le foin. La fleur de papier rentre dans la poche. Une poudre jaune dort sur l'herbe. On rentre, Aniss. Le portail de bois cliquette, tout seul.</t>
+          <t>Le papillon jaune se pose, au bout d'une tige. Mes bras ont fait des ailes. Les miennes aussi, tout lent. Vous avez marché à son pas. Le pré sent encore le foin. La fleur de papier rentre dans la poche. Une poudre jaune dort sur l'herbe. Il est venu, Aniss. Le portail de bois cliquette, tout seul.</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Le papillon jaune se pose, au bout d'une tige. On a marché, chacun son tour. Tu battais des bras, moi j'avançais. Vous avez laissé l'élan dessiner. Le pré sent encore le foin. La fleur de papier rentre dans la poche. Une poudre jaune dort sur l'herbe. On rentre, Aniss. Le portail de bois cliquette, tout seul.</t>
+          <t>Le papillon jaune se pose, au bout d'une tige. Mes bras ont fait des ailes. Les miennes aussi, tout lent. Vous avez marché à son pas. Le pré sent encore le foin. La fleur de papier rentre dans la poche. Une poudre jaune dort sur l'herbe. Il est venu, Aniss. Le portail de bois cliquette, tout seul.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -12996,13 +12996,13 @@
       <c r="AW67" t="inlineStr">
         <is>
           <t>narrateur|Le papillon jaune se pose, au bout d'une tige.
-copain|On a marché, chacun son tour.
-enfant-m|Tu battais des bras, moi j'avançais.
-papa|Vous avez laissé l'élan dessiner.
+copain|Mes bras ont fait des ailes.
+enfant-m|Les miennes aussi, tout lent.
+papa|Vous avez marché à son pas.
 maman|Le pré sent encore le foin.
 narrateur|La fleur de papier rentre dans la poche.
 narrateur|Une poudre jaune dort sur l'herbe.
-enfant-m|On rentre, Aniss.
+enfant-m|Il est venu, Aniss.
 narrateur|Le portail de bois cliquette, tout seul.</t>
         </is>
       </c>
@@ -13030,12 +13030,12 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>On s'assoit un peu. Je m'assois, alors. Aniss pose les genoux dans l'herbe. La fleur de papier attend près des genoux. Sa respiration redevient calme, tout doux. Tu es prêt ? Je ne cours plus. Vous avez laissé l'élan s'asseoir. Le pré vous a gardés.</t>
+          <t>On s'assoit un peu. Je m'assois, alors. Aniss pose les genoux dans l'herbe. La fleur de papier tient entre deux paumes. Une tige se redresse, tout contre sa chaussure. Tu es prêt ? Je ne cours plus. Vous avez attendu l'herbe. Le jaune peut redescendre, maintenant.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>On s'assoit un peu. Je m'assois, alors. Aniss pose les genoux dans l'herbe. La fleur de papier attend près des genoux. Sa respiration redevient calme, tout doux. Tu es prêt ? Je ne cours plus. Vous avez laissé l'élan s'asseoir. Le pré vous a gardés.</t>
+          <t>On s'assoit un peu. Je m'assois, alors. Aniss pose les genoux dans l'herbe. La fleur de papier tient entre deux paumes. Une tige se redresse, tout contre sa chaussure. Tu es prêt ? Je ne cours plus. Vous avez attendu l'herbe. Le jaune peut redescendre, maintenant.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13173,12 +13173,12 @@
           <t>enfant-m|On s'assoit un peu.
 copain|Je m'assois, alors.
 narrateur|Aniss pose les genoux dans l'herbe.
-narrateur|La fleur de papier attend près des genoux.
-narrateur|Sa respiration redevient calme, tout doux.
+narrateur|La fleur de papier tient entre deux paumes.
+narrateur|Une tige se redresse, tout contre sa chaussure.
 enfant-m|Tu es prêt ?
 copain|Je ne cours plus.
-papa|Vous avez laissé l'élan s'asseoir.
-maman|Le pré vous a gardés.</t>
+papa|Vous avez attendu l'herbe.
+maman|Le jaune peut redescendre, maintenant.</t>
         </is>
       </c>
     </row>
@@ -13205,12 +13205,12 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>L'herbe garde encore la chaleur des genoux. Tu t'es assis, d'abord. Puis le jaune est venu, tout droit. L'élan s'est assis, puis il a guetté. Le pré redevient calme. La fleur de papier rentre dans la poche. Une graine reste coincée au tissu. À demain, les tiges. Le gravier du chemin brille un peu.</t>
+          <t>L'herbe garde encore la chaleur des genoux. Tu t'es assis, d'abord. Puis le jaune est venu, tout droit. Vous avez attendu, assis. Une tige vous a chatouillés, sans rien dire. La fleur de papier rentre dans la poche. Une graine reste coincée au tissu. À demain, les tiges. Le gravier du chemin brille un peu.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>L'herbe garde encore la chaleur des genoux. Tu t'es assis, d'abord. Puis le jaune est venu, tout droit. L'élan s'est assis, puis il a guetté. Le pré redevient calme. La fleur de papier rentre dans la poche. Une graine reste coincée au tissu. À demain, les tiges. Le gravier du chemin brille un peu.</t>
+          <t>L'herbe garde encore la chaleur des genoux. Tu t'es assis, d'abord. Puis le jaune est venu, tout droit. Vous avez attendu, assis. Une tige vous a chatouillés, sans rien dire. La fleur de papier rentre dans la poche. Une graine reste coincée au tissu. À demain, les tiges. Le gravier du chemin brille un peu.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -13348,8 +13348,8 @@
           <t>narrateur|L'herbe garde encore la chaleur des genoux.
 enfant-m|Tu t'es assis, d'abord.
 copain|Puis le jaune est venu, tout droit.
-papa|L'élan s'est assis, puis il a guetté.
-maman|Le pré redevient calme.
+papa|Vous avez attendu, assis.
+maman|Une tige vous a chatouillés, sans rien dire.
 narrateur|La fleur de papier rentre dans la poche.
 narrateur|Une graine reste coincée au tissu.
 enfant-m|À demain, les tiges.
@@ -13380,12 +13380,12 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu restes avec nous ? Un, deux, trois, on ne bouge plus. Aniss s'arrête seulement quand elle dit trois. Victorino lève la fleur à chaque chiffre. Je peux attendre le trois ! Moi aussi, j'attends. L'herbe redevient droite, autour. Vous avez demandé, et ça marche. Mes chiffres ont tenu l'élan.</t>
+          <t>Maman, tu restes avec nous ? Chut, on écoute l'herbe. Aniss ouvre la bouche, puis la referme. Victorino tient la fleur, sans la secouer. Je peux être silencieux ! Moi aussi, j'écoute. Un criquet reprend, tout près. Vous avez demandé, et ça tient. Mon chut a tenu vos pieds.</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu restes avec nous ? Un, deux, trois, on ne bouge plus. Aniss s'arrête seulement quand elle dit trois. Victorino lève la fleur à chaque chiffre. Je peux attendre le trois ! Moi aussi, j'attends. L'herbe redevient droite, autour. Vous avez demandé, et ça marche. Mes chiffres ont tenu l'élan.</t>
+          <t>Maman, tu restes avec nous ? Chut, on écoute l'herbe. Aniss ouvre la bouche, puis la referme. Victorino tient la fleur, sans la secouer. Je peux être silencieux ! Moi aussi, j'écoute. Un criquet reprend, tout près. Vous avez demandé, et ça tient. Mon chut a tenu vos pieds.</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -13521,14 +13521,14 @@
       <c r="AW70" t="inlineStr">
         <is>
           <t>enfant-m|Maman, tu restes avec nous ?
-maman|Un, deux, trois, on ne bouge plus.
-narrateur|Aniss s'arrête seulement quand elle dit trois.
-narrateur|Victorino lève la fleur à chaque chiffre.
-copain|Je peux attendre le trois !
-enfant-m|Moi aussi, j'attends.
-narrateur|L'herbe redevient droite, autour.
-papa|Vous avez demandé, et ça marche.
-maman|Mes chiffres ont tenu l'élan.</t>
+maman|Chut, on écoute l'herbe.
+narrateur|Aniss ouvre la bouche, puis la referme.
+narrateur|Victorino tient la fleur, sans la secouer.
+copain|Je peux être silencieux !
+enfant-m|Moi aussi, j'écoute.
+narrateur|Un criquet reprend, tout près.
+papa|Vous avez demandé, et ça tient.
+maman|Mon chut a tenu vos pieds.</t>
         </is>
       </c>
     </row>
@@ -13555,12 +13555,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Le trois de maman reste dans l'air, tout léger. J'ai attendu le chiffre. On a demandé, et ça allait. Mes mots ont tenu vos pieds. Le pré vous rend le silence. La fleur de papier pose un grain de jaune sur le bois. Victorino touche la tige, du bout. Il s'est posé. Une ombre de peuplier barre encore l'herbe.</t>
+          <t>Le chut de maman reste dans l'air, tout léger. J'ai fermé la bouche. On a demandé, et ça tenait. Mon silence a tenu vos pieds. Le criquet a repris, pour vous. La fleur de papier pose un grain de jaune sur le bois. Victorino touche la tige, du bout. Il s'est posé. Une ombre de peuplier barre encore l'herbe.</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>Le trois de maman reste dans l'air, tout léger. J'ai attendu le chiffre. On a demandé, et ça allait. Mes mots ont tenu vos pieds. Le pré vous rend le silence. La fleur de papier pose un grain de jaune sur le bois. Victorino touche la tige, du bout. Il s'est posé. Une ombre de peuplier barre encore l'herbe.</t>
+          <t>Le chut de maman reste dans l'air, tout léger. J'ai fermé la bouche. On a demandé, et ça tenait. Mon silence a tenu vos pieds. Le criquet a repris, pour vous. La fleur de papier pose un grain de jaune sur le bois. Victorino touche la tige, du bout. Il s'est posé. Une ombre de peuplier barre encore l'herbe.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -13695,11 +13695,11 @@
       <c r="AV71" s="2" t="inlineStr"/>
       <c r="AW71" t="inlineStr">
         <is>
-          <t>narrateur|Le trois de maman reste dans l'air, tout léger.
-copain|J'ai attendu le chiffre.
-enfant-m|On a demandé, et ça allait.
-maman|Mes mots ont tenu vos pieds.
-papa|Le pré vous rend le silence.
+          <t>narrateur|Le chut de maman reste dans l'air, tout léger.
+copain|J'ai fermé la bouche.
+enfant-m|On a demandé, et ça tenait.
+maman|Mon silence a tenu vos pieds.
+papa|Le criquet a repris, pour vous.
 narrateur|La fleur de papier pose un grain de jaune sur le bois.
 narrateur|Victorino touche la tige, du bout.
 copain|Il s'est posé.
@@ -13730,12 +13730,12 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Victorino tend la fleur vers le violet. Les lavandes sentent partout, Aniss. Je vais jusqu'au bout, trop vite ! Ses pieds tapent les tiges, puis reviennent. Un coude plie le papier, trop fort. Un parfum lève, puis retombe. Il a de l'élan, comme un petit vent. Toi tu vas plus loin, lui plus vite. On peut guetter avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Victorino tend la fleur vers le violet. Ça sent le savon et le miel, Aniss. Je pousse les tiges, trop fort ! Un nuage de parfum saute, puis retombe. Un coude plie le papier, trop fort. Le jaune quitte le violet, d'un coup. Tes pieds ont réveillé les fleurs. On s'approche sans les bousculer. Il peut revenir ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>Victorino tend la fleur vers le violet. Les lavandes sentent partout, Aniss. Je vais jusqu'au bout, trop vite ! Ses pieds tapent les tiges, puis reviennent. Un coude plie le papier, trop fort. Un parfum lève, puis retombe. Il a de l'élan, comme un petit vent. Toi tu vas plus loin, lui plus vite. On peut guetter avec lui ? Vous trouvez, tous les deux ?</t>
+          <t>Victorino tend la fleur vers le violet. Ça sent le savon et le miel, Aniss. Je pousse les tiges, trop fort ! Un nuage de parfum saute, puis retombe. Un coude plie le papier, trop fort. Le jaune quitte le violet, d'un coup. Tes pieds ont réveillé les fleurs. On s'approche sans les bousculer. Il peut revenir ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -13871,14 +13871,14 @@
       <c r="AW72" t="inlineStr">
         <is>
           <t>narrateur|Victorino tend la fleur vers le violet.
-enfant-m|Les lavandes sentent partout, Aniss.
-copain|Je vais jusqu'au bout, trop vite !
-narrateur|Ses pieds tapent les tiges, puis reviennent.
+enfant-m|Ça sent le savon et le miel, Aniss.
+copain|Je pousse les tiges, trop fort !
+narrateur|Un nuage de parfum saute, puis retombe.
 narrateur|Un coude plie le papier, trop fort.
-narrateur|Un parfum lève, puis retombe.
-maman|Il a de l'élan, comme un petit vent.
-papa|Toi tu vas plus loin, lui plus vite.
-enfant-m|On peut guetter avec lui ?
+narrateur|Le jaune quitte le violet, d'un coup.
+maman|Tes pieds ont réveillé les fleurs.
+papa|On s'approche sans les bousculer.
+enfant-m|Il peut revenir ?
 papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
@@ -13911,12 +13911,12 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Les lavandes bougent encore, un peu. Souffler, attendre, ou la fleur de papa ?</t>
+          <t>Le parfum tient encore, tout bas. Souffler, attendre, ou la fleur de papa ?</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Les lavandes bougent encore, un peu. Souffler, attendre, ou la fleur de papa ?</t>
+          <t>Le parfum tient encore, tout bas. Souffler, attendre, ou la fleur de papa ?</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -14075,7 +14075,7 @@
       <c r="AV73" s="2" t="inlineStr"/>
       <c r="AW73" t="inlineStr">
         <is>
-          <t>narrateur|Les lavandes bougent encore, un peu.
+          <t>narrateur|Le parfum tient encore, tout bas.
 maman|Souffler, attendre, ou la fleur de papa ?</t>
         </is>
       </c>
@@ -14103,12 +14103,12 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>On souffle tout doux. Toi derrière, moi devant ! Victorino garde la fleur, Aniss souffle devant. Deux souffles passent sur la même tige. Aniss va plus vite, Victorino plus loin. On arrive au violet, tous les deux. J'ai attendu ton souffle, un peu. Vous avez joué avec l'élan. Les lavandes vous ont laissés passer.</t>
+          <t>On souffle tout doux. Comme le petit vent ! Victorino garde la fleur, Aniss souffle devant. Deux souffles passent sur la même tige. Le violet penche, puis se redresse. On n'a rien cassé. J'ai soufflé plus bas, cette fois. Vous avez joué avec l'air. Les fleurs sont restées debout.</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>On souffle tout doux. Toi derrière, moi devant ! Victorino garde la fleur, Aniss souffle devant. Deux souffles passent sur la même tige. Aniss va plus vite, Victorino plus loin. On arrive au violet, tous les deux. J'ai attendu ton souffle, un peu. Vous avez joué avec l'élan. Les lavandes vous ont laissés passer.</t>
+          <t>On souffle tout doux. Comme le petit vent ! Victorino garde la fleur, Aniss souffle devant. Deux souffles passent sur la même tige. Le violet penche, puis se redresse. On n'a rien cassé. J'ai soufflé plus bas, cette fois. Vous avez joué avec l'air. Les fleurs sont restées debout.</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -14244,14 +14244,14 @@
       <c r="AW74" t="inlineStr">
         <is>
           <t>enfant-m|On souffle tout doux.
-copain|Toi derrière, moi devant !
+copain|Comme le petit vent !
 narrateur|Victorino garde la fleur, Aniss souffle devant.
 narrateur|Deux souffles passent sur la même tige.
-narrateur|Aniss va plus vite, Victorino plus loin.
-enfant-m|On arrive au violet, tous les deux.
-copain|J'ai attendu ton souffle, un peu.
-papa|Vous avez joué avec l'élan.
-maman|Les lavandes vous ont laissés passer.</t>
+narrateur|Le violet penche, puis se redresse.
+enfant-m|On n'a rien cassé.
+copain|J'ai soufflé plus bas, cette fois.
+papa|Vous avez joué avec l'air.
+maman|Les fleurs sont restées debout.</t>
         </is>
       </c>
     </row>
@@ -14278,12 +14278,12 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Deux souffles marquent la même tige violette. Toi devant, moi derrière. Tes pas allaient plus loin. Vous avez soufflé avec l'élan, pas contre. Les lavandes redeviennent tièdes, et calmes. La fleur de papier rentre dans la poche. Un brin violet sèche déjà sur le tissu. On rentre, le parfum reste. Le puits fait une ombre ronde.</t>
+          <t>Deux souffles marquent la même tige violette. On n'a rien cassé. J'ai soufflé plus bas. Vous avez joué avec l'air. Les lavandes sont encore debout. La fleur de papier rentre dans la poche. Un brin violet sèche déjà sur le tissu. Le parfum rentre avec nous. Le puits fait une ombre ronde.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Deux souffles marquent la même tige violette. Toi devant, moi derrière. Tes pas allaient plus loin. Vous avez soufflé avec l'élan, pas contre. Les lavandes redeviennent tièdes, et calmes. La fleur de papier rentre dans la poche. Un brin violet sèche déjà sur le tissu. On rentre, le parfum reste. Le puits fait une ombre ronde.</t>
+          <t>Deux souffles marquent la même tige violette. On n'a rien cassé. J'ai soufflé plus bas. Vous avez joué avec l'air. Les lavandes sont encore debout. La fleur de papier rentre dans la poche. Un brin violet sèche déjà sur le tissu. Le parfum rentre avec nous. Le puits fait une ombre ronde.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -14419,13 +14419,13 @@
       <c r="AW75" t="inlineStr">
         <is>
           <t>narrateur|Deux souffles marquent la même tige violette.
-enfant-m|Toi devant, moi derrière.
-copain|Tes pas allaient plus loin.
-papa|Vous avez soufflé avec l'élan, pas contre.
-maman|Les lavandes redeviennent tièdes, et calmes.
+enfant-m|On n'a rien cassé.
+copain|J'ai soufflé plus bas.
+papa|Vous avez joué avec l'air.
+maman|Les lavandes sont encore debout.
 narrateur|La fleur de papier rentre dans la poche.
 narrateur|Un brin violet sèche déjà sur le tissu.
-enfant-m|On rentre, le parfum reste.
+enfant-m|Le parfum rentre avec nous.
 narrateur|Le puits fait une ombre ronde.</t>
         </is>
       </c>
@@ -14453,12 +14453,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>J'attends le parfum. Moi je finis, puis c'est toi. Victorino tient la fleur, sans la bouger. Aniss tapote une tige, tout seul d'abord. Il souffle, puis il recule. C'est à toi, Victorino. Merci, j'y vais. Chacun son tour, entre les tiges. L'élan a attendu le parfum.</t>
+          <t>J'attends le parfum. Quand il retombe, on avance. Victorino tient la fleur, sans la bouger. Aniss compte les tiges, tout bas. Le nuage violet s'assoit, enfin. C'est à toi, Victorino. Merci, j'y vais. Le parfum vous a fait de la place. Vous l'avez laissé se poser.</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>J'attends le parfum. Moi je finis, puis c'est toi. Victorino tient la fleur, sans la bouger. Aniss tapote une tige, tout seul d'abord. Il souffle, puis il recule. C'est à toi, Victorino. Merci, j'y vais. Chacun son tour, entre les tiges. L'élan a attendu le parfum.</t>
+          <t>J'attends le parfum. Quand il retombe, on avance. Victorino tient la fleur, sans la bouger. Aniss compte les tiges, tout bas. Le nuage violet s'assoit, enfin. C'est à toi, Victorino. Merci, j'y vais. Le parfum vous a fait de la place. Vous l'avez laissé se poser.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -14594,14 +14594,14 @@
       <c r="AW76" t="inlineStr">
         <is>
           <t>enfant-m|J'attends le parfum.
-copain|Moi je finis, puis c'est toi.
+copain|Quand il retombe, on avance.
 narrateur|Victorino tient la fleur, sans la bouger.
-narrateur|Aniss tapote une tige, tout seul d'abord.
-narrateur|Il souffle, puis il recule.
+narrateur|Aniss compte les tiges, tout bas.
+narrateur|Le nuage violet s'assoit, enfin.
 copain|C'est à toi, Victorino.
 enfant-m|Merci, j'y vais.
-papa|Chacun son tour, entre les tiges.
-maman|L'élan a attendu le parfum.</t>
+papa|Le parfum vous a fait de la place.
+maman|Vous l'avez laissé se poser.</t>
         </is>
       </c>
     </row>
@@ -14628,12 +14628,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Le parfum attend encore, tout bas. J'ai fini, puis c'était toi. J'ai attendu ta tige. Chacun son tour, entre les tiges. L'élan a laissé la place. La fleur de papier garde un grain de parfum. Victorino souffle dessus, tout doux. On se dit au revoir, lavandes. Une abeille passe, sans se presser.</t>
+          <t>Le parfum s'est assis, tout bas. Quand il est retombé, on a avancé. J'ai attendu ta tige. Le nuage vous a laissés passer. Vous l'avez laissé se poser. La fleur de papier garde un grain de parfum. Victorino souffle dessus, tout doux. Au revoir, les tiges. Une abeille passe, sans se presser.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Le parfum attend encore, tout bas. J'ai fini, puis c'était toi. J'ai attendu ta tige. Chacun son tour, entre les tiges. L'élan a laissé la place. La fleur de papier garde un grain de parfum. Victorino souffle dessus, tout doux. On se dit au revoir, lavandes. Une abeille passe, sans se presser.</t>
+          <t>Le parfum s'est assis, tout bas. Quand il est retombé, on a avancé. J'ai attendu ta tige. Le nuage vous a laissés passer. Vous l'avez laissé se poser. La fleur de papier garde un grain de parfum. Victorino souffle dessus, tout doux. Au revoir, les tiges. Une abeille passe, sans se presser.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -14768,14 +14768,14 @@
       <c r="AV77" s="2" t="inlineStr"/>
       <c r="AW77" t="inlineStr">
         <is>
-          <t>narrateur|Le parfum attend encore, tout bas.
-copain|J'ai fini, puis c'était toi.
+          <t>narrateur|Le parfum s'est assis, tout bas.
+copain|Quand il est retombé, on a avancé.
 enfant-m|J'ai attendu ta tige.
-maman|Chacun son tour, entre les tiges.
-papa|L'élan a laissé la place.
+maman|Le nuage vous a laissés passer.
+papa|Vous l'avez laissé se poser.
 narrateur|La fleur de papier garde un grain de parfum.
 narrateur|Victorino souffle dessus, tout doux.
-copain|On se dit au revoir, lavandes.
+copain|Au revoir, les tiges.
 narrateur|Une abeille passe, sans se presser.</t>
         </is>
       </c>
@@ -14803,12 +14803,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu gardes la fleur ? Je la tends, un pas chacun. Papa pose la fleur dans sa paume. Aniss s'approche, tout petit pas. Victorino s'approche, encore plus lent. On demande, et ça va ! Le violet est à nous. Vous avez demandé, tout calme. Ma main a juste attendu.</t>
+          <t>Papa, tu gardes la fleur ? Je la tends, un pas chacun. Papa pose la fleur dans sa paume. Aniss pose un pied, puis l'autre. Victorino pose le même pas, plus tard. On a demandé, et ça va ! Le violet est tout près. Vous avez demandé, tout calme. Ma main n'a pas bougé.</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Papa, tu gardes la fleur ? Je la tends, un pas chacun. Papa pose la fleur dans sa paume. Aniss s'approche, tout petit pas. Victorino s'approche, encore plus lent. On demande, et ça va ! Le violet est à nous. Vous avez demandé, tout calme. Ma main a juste attendu.</t>
+          <t>Papa, tu gardes la fleur ? Je la tends, un pas chacun. Papa pose la fleur dans sa paume. Aniss pose un pied, puis l'autre. Victorino pose le même pas, plus tard. On a demandé, et ça va ! Le violet est tout près. Vous avez demandé, tout calme. Ma main n'a pas bougé.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -14946,12 +14946,12 @@
           <t>enfant-m|Papa, tu gardes la fleur ?
 papa|Je la tends, un pas chacun.
 narrateur|Papa pose la fleur dans sa paume.
-narrateur|Aniss s'approche, tout petit pas.
-narrateur|Victorino s'approche, encore plus lent.
-copain|On demande, et ça va !
-enfant-m|Le violet est à nous.
+narrateur|Aniss pose un pied, puis l'autre.
+narrateur|Victorino pose le même pas, plus tard.
+copain|On a demandé, et ça va !
+enfant-m|Le violet est tout près.
 maman|Vous avez demandé, tout calme.
-papa|Ma main a juste attendu.</t>
+papa|Ma main n'a pas bougé.</t>
         </is>
       </c>
     </row>
@@ -14978,12 +14978,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>La fleur de papa repose près du violet. Tu la tendais, un pas chacun. On a demandé, et ça venait juste. Ma main a fait le tour, rien de plus. Les lavandes ont rendu le jaune. La fleur de papier rentre dans la poche. Un rond clair reste sur une feuille. Regarde, Aniss, il brille. Le chat reprend la pierre, au frais.</t>
+          <t>La fleur de papa repose près du violet. Tu la tendais, un pas chacun. On a demandé, et ça venait juste. Ma main n'a pas bougé. Les lavandes ont rendu le jaune. La fleur de papier rentre dans la poche. Un rond clair reste sur une feuille. Regarde, Aniss, il brille. Le chat reprend la pierre, au frais.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>La fleur de papa repose près du violet. Tu la tendais, un pas chacun. On a demandé, et ça venait juste. Ma main a fait le tour, rien de plus. Les lavandes ont rendu le jaune. La fleur de papier rentre dans la poche. Un rond clair reste sur une feuille. Regarde, Aniss, il brille. Le chat reprend la pierre, au frais.</t>
+          <t>La fleur de papa repose près du violet. Tu la tendais, un pas chacun. On a demandé, et ça venait juste. Ma main n'a pas bougé. Les lavandes ont rendu le jaune. La fleur de papier rentre dans la poche. Un rond clair reste sur une feuille. Regarde, Aniss, il brille. Le chat reprend la pierre, au frais.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -15121,7 +15121,7 @@
           <t>narrateur|La fleur de papa repose près du violet.
 enfant-m|Tu la tendais, un pas chacun.
 copain|On a demandé, et ça venait juste.
-papa|Ma main a fait le tour, rien de plus.
+papa|Ma main n'a pas bougé.
 maman|Les lavandes ont rendu le jaune.
 narrateur|La fleur de papier rentre dans la poche.
 narrateur|Un rond clair reste sur une feuille.
@@ -15153,12 +15153,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>La fleur de papier attend sur la pierre. Ici, la pierre est chaude, Aniss. J'entends mes pieds deux fois ! Le muret renvoie chaque pas, tout fort. La fleur glisse dans une fente. La fleur de papier attend au bord, un peu seule. Son élan remplit toute la pierre. Toi tu vas plus loin, lui plus vite. On guette comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>La fleur de papier attend sur la pierre. La pierre est tiède, Aniss. J'entends mes pieds deux fois ! Chaque clic revient, plus fort. La fleur glisse dans une fente. La fleur de papier n'ose plus bouger. Le jaune n'aime pas le bruit. La pierre répète tes pas. On fait moins de clic ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>La fleur de papier attend sur la pierre. Ici, la pierre est chaude, Aniss. J'entends mes pieds deux fois ! Le muret renvoie chaque pas, tout fort. La fleur glisse dans une fente. La fleur de papier attend au bord, un peu seule. Son élan remplit toute la pierre. Toi tu vas plus loin, lui plus vite. On guette comment, alors ? Vous trouvez, tous les deux ?</t>
+          <t>La fleur de papier attend sur la pierre. La pierre est tiède, Aniss. J'entends mes pieds deux fois ! Chaque clic revient, plus fort. La fleur glisse dans une fente. La fleur de papier n'ose plus bouger. Le jaune n'aime pas le bruit. La pierre répète tes pas. On fait moins de clic ? Vous trouvez, tous les deux ?</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -15294,14 +15294,14 @@
       <c r="AW80" t="inlineStr">
         <is>
           <t>narrateur|La fleur de papier attend sur la pierre.
-enfant-m|Ici, la pierre est chaude, Aniss.
+enfant-m|La pierre est tiède, Aniss.
 copain|J'entends mes pieds deux fois !
-narrateur|Le muret renvoie chaque pas, tout fort.
+narrateur|Chaque clic revient, plus fort.
 narrateur|La fleur glisse dans une fente.
-narrateur|La fleur de papier attend au bord, un peu seule.
-maman|Son élan remplit toute la pierre.
-papa|Toi tu vas plus loin, lui plus vite.
-copain|On guette comment, alors ?
+narrateur|La fleur de papier n'ose plus bouger.
+maman|Le jaune n'aime pas le bruit.
+papa|La pierre répète tes pas.
+copain|On fait moins de clic ?
 papa|Vous trouvez, tous les deux ?</t>
         </is>
       </c>
@@ -15329,12 +15329,12 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Les clics remplissent encore le muret. Le rythme, en bas, ou la main de maman ?</t>
+          <t>Un dernier clic roule le long du muret. Le rythme, en bas, ou la main de maman ?</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Les clics remplissent encore le muret. Le rythme, en bas, ou la main de maman ?</t>
+          <t>Un dernier clic roule le long du muret. Le rythme, en bas, ou la main de maman ?</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -15493,7 +15493,7 @@
       <c r="AV81" s="2" t="inlineStr"/>
       <c r="AW81" t="inlineStr">
         <is>
-          <t>narrateur|Les clics remplissent encore le muret.
+          <t>narrateur|Un dernier clic roule le long du muret.
 papa|Le rythme, en bas, ou la main de maman ?</t>
         </is>
       </c>
@@ -15521,12 +15521,12 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>On fait un rythme sur la pierre. Toc toc, j'avance ! Victorino pose une main sur l'épaule d'Aniss. La fleur de papier voyage sur la pierre, entre deux taps. Ils tapent la même pierre, l'un après l'autre. Doucement, le rythme tient. Le clic suit le rythme, puis se tait. Vous jouez avec le bruit, ensemble. Le muret est devenu un tambour.</t>
+          <t>On tape une fois, puis plus. Toc, et j'attends. Victorino pose une main sur l'épaule d'Aniss. La fleur de papier s'arrête après le dernier toc. La pierre répond, puis se tait. Le jaune aime le silence, après. Moi aussi, après le toc. Vous avez joué avec le bruit. Un toc, puis la pierre dort.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>On fait un rythme sur la pierre. Toc toc, j'avance ! Victorino pose une main sur l'épaule d'Aniss. La fleur de papier voyage sur la pierre, entre deux taps. Ils tapent la même pierre, l'un après l'autre. Doucement, le rythme tient. Le clic suit le rythme, puis se tait. Vous jouez avec le bruit, ensemble. Le muret est devenu un tambour.</t>
+          <t>On tape une fois, puis plus. Toc, et j'attends. Victorino pose une main sur l'épaule d'Aniss. La fleur de papier s'arrête après le dernier toc. La pierre répond, puis se tait. Le jaune aime le silence, après. Moi aussi, après le toc. Vous avez joué avec le bruit. Un toc, puis la pierre dort.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -15661,15 +15661,15 @@
       <c r="AV82" s="2" t="inlineStr"/>
       <c r="AW82" t="inlineStr">
         <is>
-          <t>enfant-m|On fait un rythme sur la pierre.
-copain|Toc toc, j'avance !
+          <t>enfant-m|On tape une fois, puis plus.
+copain|Toc, et j'attends.
 narrateur|Victorino pose une main sur l'épaule d'Aniss.
-narrateur|La fleur de papier voyage sur la pierre, entre deux taps.
-narrateur|Ils tapent la même pierre, l'un après l'autre.
-enfant-m|Doucement, le rythme tient.
-copain|Le clic suit le rythme, puis se tait.
-papa|Vous jouez avec le bruit, ensemble.
-maman|Le muret est devenu un tambour.</t>
+narrateur|La fleur de papier s'arrête après le dernier toc.
+narrateur|La pierre répond, puis se tait.
+enfant-m|Le jaune aime le silence, après.
+copain|Moi aussi, après le toc.
+papa|Vous avez joué avec le bruit.
+maman|Un toc, puis la pierre dort.</t>
         </is>
       </c>
     </row>
@@ -15696,12 +15696,12 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Le rythme s'arrête, et le jaune se pose. Toc toc, on est arrivés. J'avais la main sur ton épaule. Le muret est redevenu une pierre, simplement. Le clic s'est couché. La fleur de papier rentre dans la poche. Une poussière tourne encore, puis tombe. On rentre, le tambour se tait. Dehors, le pré redevient calme.</t>
+          <t>Après le toc, le jaune se pose. J'ai tapé une fois, puis plus. J'avais la main sur ton épaule. La pierre a fini par dormir. Un toc, puis le silence. La fleur de papier rentre dans la poche. Une poussière tourne encore, puis tombe. Le muret s'est tu. Dehors, le pré redevient calme.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Le rythme s'arrête, et le jaune se pose. Toc toc, on est arrivés. J'avais la main sur ton épaule. Le muret est redevenu une pierre, simplement. Le clic s'est couché. La fleur de papier rentre dans la poche. Une poussière tourne encore, puis tombe. On rentre, le tambour se tait. Dehors, le pré redevient calme.</t>
+          <t>Après le toc, le jaune se pose. J'ai tapé une fois, puis plus. J'avais la main sur ton épaule. La pierre a fini par dormir. Un toc, puis le silence. La fleur de papier rentre dans la poche. Une poussière tourne encore, puis tombe. Le muret s'est tu. Dehors, le pré redevient calme.</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -15836,14 +15836,14 @@
       <c r="AV83" s="2" t="inlineStr"/>
       <c r="AW83" t="inlineStr">
         <is>
-          <t>narrateur|Le rythme s'arrête, et le jaune se pose.
-copain|Toc toc, on est arrivés.
+          <t>narrateur|Après le toc, le jaune se pose.
+copain|J'ai tapé une fois, puis plus.
 enfant-m|J'avais la main sur ton épaule.
-papa|Le muret est redevenu une pierre, simplement.
-maman|Le clic s'est couché.
+papa|La pierre a fini par dormir.
+maman|Un toc, puis le silence.
 narrateur|La fleur de papier rentre dans la poche.
 narrateur|Une poussière tourne encore, puis tombe.
-enfant-m|On rentre, le tambour se tait.
+enfant-m|Le muret s'est tu.
 narrateur|Dehors, le pré redevient calme.</t>
         </is>
       </c>
@@ -15871,12 +15871,12 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>On attend en bas. Quand la pierre se tait, je m'approche. Un pas dans l'herbe, puis plus rien. La fleur de papier reste muette, au creux. Le muret se tait, enfin. Maintenant ! À toi, puis à moi. Vous avez laissé le bruit s'asseoir. L'élan a attendu le silence.</t>
+          <t>On attend en bas. La pierre se tait, d'abord. Leurs chaussures restent dans l'herbe fraîche. La fleur de papier reste dans l'herbe, en bas. Le muret ne clique plus. Maintenant, on peut regarder. À toi, puis à moi. Vous avez laissé le bruit s'en aller. En bas, vos pieds sont plus doux.</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>On attend en bas. Quand la pierre se tait, je m'approche. Un pas dans l'herbe, puis plus rien. La fleur de papier reste muette, au creux. Le muret se tait, enfin. Maintenant ! À toi, puis à moi. Vous avez laissé le bruit s'asseoir. L'élan a attendu le silence.</t>
+          <t>On attend en bas. La pierre se tait, d'abord. Leurs chaussures restent dans l'herbe fraîche. La fleur de papier reste dans l'herbe, en bas. Le muret ne clique plus. Maintenant, on peut regarder. À toi, puis à moi. Vous avez laissé le bruit s'en aller. En bas, vos pieds sont plus doux.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -16012,14 +16012,14 @@
       <c r="AW84" t="inlineStr">
         <is>
           <t>enfant-m|On attend en bas.
-copain|Quand la pierre se tait, je m'approche.
-narrateur|Un pas dans l'herbe, puis plus rien.
-narrateur|La fleur de papier reste muette, au creux.
-narrateur|Le muret se tait, enfin.
-copain|Maintenant !
+copain|La pierre se tait, d'abord.
+narrateur|Leurs chaussures restent dans l'herbe fraîche.
+narrateur|La fleur de papier reste dans l'herbe, en bas.
+narrateur|Le muret ne clique plus.
+copain|Maintenant, on peut regarder.
 enfant-m|À toi, puis à moi.
-papa|Vous avez laissé le bruit s'asseoir.
-maman|L'élan a attendu le silence.</t>
+papa|Vous avez laissé le bruit s'en aller.
+maman|En bas, vos pieds sont plus doux.</t>
         </is>
       </c>
     </row>
@@ -16046,12 +16046,12 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>La pierre s'est tue, enfin, tout à fait. On a attendu en bas. Quand elle était partie, on s'approchait. Le silence vous a laissé le jaune. L'élan a écouté la pierre. La fleur de papier ne fait plus aucun bruit. Victorino pose la paume sur la pierre chaude. Elle est tiède. Un oiseau passe au-dessus du muret, sans crier.</t>
+          <t>La pierre s'est tue, enfin, tout à fait. On a attendu en bas. Nos chaussures sont restées dans l'herbe. Le silence vous a laissé le jaune. En bas, vos pieds étaient plus doux. La fleur de papier ne fait plus aucun bruit. Victorino pose la paume sur la pierre chaude. Elle est tiède. Un oiseau passe au-dessus du muret, sans crier.</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>La pierre s'est tue, enfin, tout à fait. On a attendu en bas. Quand elle était partie, on s'approchait. Le silence vous a laissé le jaune. L'élan a écouté la pierre. La fleur de papier ne fait plus aucun bruit. Victorino pose la paume sur la pierre chaude. Elle est tiède. Un oiseau passe au-dessus du muret, sans crier.</t>
+          <t>La pierre s'est tue, enfin, tout à fait. On a attendu en bas. Nos chaussures sont restées dans l'herbe. Le silence vous a laissé le jaune. En bas, vos pieds étaient plus doux. La fleur de papier ne fait plus aucun bruit. Victorino pose la paume sur la pierre chaude. Elle est tiède. Un oiseau passe au-dessus du muret, sans crier.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -16188,9 +16188,9 @@
         <is>
           <t>narrateur|La pierre s'est tue, enfin, tout à fait.
 enfant-m|On a attendu en bas.
-copain|Quand elle était partie, on s'approchait.
+copain|Nos chaussures sont restées dans l'herbe.
 papa|Le silence vous a laissé le jaune.
-maman|L'élan a écouté la pierre.
+maman|En bas, vos pieds étaient plus doux.
 narrateur|La fleur de papier ne fait plus aucun bruit.
 narrateur|Victorino pose la paume sur la pierre chaude.
 copain|Elle est tiède.
@@ -16221,12 +16221,12 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tends la main ? Je reste, et vous venez tout doux. Aniss écoute la paume, plus que ses pieds. Victorino lève la fleur quand maman ouvre la paume. Je m'arrête sur ta main ! Moi aussi, j'écoute. Le clic se range derrière le silence. Vous avez demandé la main. Ma paume a tenu l'élan.</t>
+          <t>Maman, tu tends la main ? Je reste, et vous venez tout doux. Aniss regarde la paume, plus que ses pieds. Victorino lève la fleur quand maman ouvre la paume. Je m'arrête devant ta main ! Moi aussi, j'écoute. Un grain de foin dort dans ses plis. Vous avez demandé la main. Ma paume est devenue une tige.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Maman, tu tends la main ? Je reste, et vous venez tout doux. Aniss écoute la paume, plus que ses pieds. Victorino lève la fleur quand maman ouvre la paume. Je m'arrête sur ta main ! Moi aussi, j'écoute. Le clic se range derrière le silence. Vous avez demandé la main. Ma paume a tenu l'élan.</t>
+          <t>Maman, tu tends la main ? Je reste, et vous venez tout doux. Aniss regarde la paume, plus que ses pieds. Victorino lève la fleur quand maman ouvre la paume. Je m'arrête devant ta main ! Moi aussi, j'écoute. Un grain de foin dort dans ses plis. Vous avez demandé la main. Ma paume est devenue une tige.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -16363,13 +16363,13 @@
         <is>
           <t>enfant-m|Maman, tu tends la main ?
 maman|Je reste, et vous venez tout doux.
-narrateur|Aniss écoute la paume, plus que ses pieds.
+narrateur|Aniss regarde la paume, plus que ses pieds.
 narrateur|Victorino lève la fleur quand maman ouvre la paume.
-copain|Je m'arrête sur ta main !
+copain|Je m'arrête devant ta main !
 enfant-m|Moi aussi, j'écoute.
-narrateur|Le clic se range derrière le silence.
+narrateur|Un grain de foin dort dans ses plis.
 papa|Vous avez demandé la main.
-maman|Ma paume a tenu l'élan.</t>
+maman|Ma paume est devenue une tige.</t>
         </is>
       </c>
     </row>
@@ -16396,12 +16396,12 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>La paume de maman s'ouvre, puis se referme. J'écoutais ta main. Moi aussi, je m'arrêtais dessus. Vous avez demandé le calme. Le muret a rendu vos pas. La fleur de papier rentre dans la poche. Victorino touche la pierre, du bout des doigts. Il s'est posé, Aniss. La pierre garde une poussière, puis plus rien.</t>
+          <t>La paume de maman s'ouvre, puis se referme. J'écoutais ta main. Moi aussi, je m'arrêtais dessus. Vous avez demandé le calme. Un grain de foin reste dans ses plis. La fleur de papier rentre dans la poche. Victorino touche la pierre, du bout des doigts. Il s'est posé, Aniss. La pierre garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>La paume de maman s'ouvre, puis se referme. J'écoutais ta main. Moi aussi, je m'arrêtais dessus. Vous avez demandé le calme. Le muret a rendu vos pas. La fleur de papier rentre dans la poche. Victorino touche la pierre, du bout des doigts. Il s'est posé, Aniss. La pierre garde une poussière, puis plus rien.</t>
+          <t>La paume de maman s'ouvre, puis se referme. J'écoutais ta main. Moi aussi, je m'arrêtais dessus. Vous avez demandé le calme. Un grain de foin reste dans ses plis. La fleur de papier rentre dans la poche. Victorino touche la pierre, du bout des doigts. Il s'est posé, Aniss. La pierre garde une poussière, puis plus rien.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -16540,7 +16540,7 @@
 enfant-m|J'écoutais ta main.
 copain|Moi aussi, je m'arrêtais dessus.
 maman|Vous avez demandé le calme.
-papa|Le muret a rendu vos pas.
+papa|Un grain de foin reste dans ses plis.
 narrateur|La fleur de papier rentre dans la poche.
 narrateur|Victorino touche la pierre, du bout des doigts.
 enfant-m|Il s'est posé, Aniss.
@@ -16565,7 +16565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16608,6 +16608,13 @@
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>